<commit_message>
Complete the claude_fp8_scratch_ten_5r record
The snapshot (804a57a) went up while the engine was still inside round 9;
this adds what finished afterwards -- round 9's judged result, round 10,
the final champion `best_workflow.json`, and the refreshed CPE state, patch
history, `results.json` and workbook exports.  Same inclusion rule as the
snapshot: round and run records only, no workspaces, solver sessions or
judge scratch files.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/workflows/interaction_evolution.xlsx
+++ b/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/workflows/interaction_evolution.xlsx
@@ -12,9 +12,9 @@
     <sheet name="轮次耗时" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'轮次策略'!$A$1:$V$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'交互历史'!$A$1:$Q$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'轮次耗时'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'轮次策略'!$A$1:$V$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'交互历史'!$A$1:$Q$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'轮次耗时'!$A$1:$K$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1973,8 +1973,148 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Mechanism-Constraint-Parameter with Anti-Prescriptive Guard</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>interaction_workflow_c83b67c63c37</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>interaction_workflow_17c7de5c9a98</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>mutation</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>## Interaction Strategy</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">【新增/改写后】
++ The consultation operates on a 'mechanism-constraint-parameter' sequence, strictly prohibiting prescriptive or 'coaching-style' questions. The agent treats the expert as a source of system dynamics and operational limits, not a strategy advisor. The hierarchy is: establish the dominant behavioral mechanism, identify the primary operational constraint, then calibrate quantitative parameters. Asking for a number before understanding the behavior and its limits is a fatal error. Asking for advice or 'what to do' is prohibited.
++ If the agent has not established the dominant behavioral mechanism or the primary causal driver, it asks for the standard operational norm or the most common real-world pattern defining how the system functions. This branch has absolute priority when the problem statement allows multiple plausible physical or logical interpretations of the core process. The agent must not assume a generic theoretical ideal; it must ask for the prevailing practice in the specific context. If two structural ambiguities exist, the agent asks about the one determining the primary state transition or main feedback loop.
++ Else, if the dominant mechanism is established but the primary operational constraint or hard limit is not, the agent asks for the specific constraint limiting the mechanism's application. This branch is critical because a mechanism without its limiting constraint leads to models assuming infinite capability. The condition is that the agent knows *how* the system acts but not *what stops it* or *what it must not violate*. The question must reference the established mechanism and ask for the specific boundary or trade-off operators must navigate.
++ Else, if the mechanism and its primary constraints are established, but the model requires a specific quantitative parameter (rate, threshold, duration, proportion) critical to dynamics and absent from the dataset, the agent asks for the typical empirical range or central estimate. This branch applies only when structural logic and constraints are fixed. The condition is that the agent knows *how* the variable acts and *what limits it*, but not *how much* it acts. The question must explicitly reference the previously established mechanism and constraint to ensure the expert calibrates the value to that specific context, not a generic textbook average. If tempted to ask for 'advice,' the agent must reframe the question into a parameter of the system's response dynamics.
++ If none of the above conditions hold, or if the agent has gathered sufficient empirical grounding for the dominant mechanism, its constraints, and critical parameters, the agent stops asking and proceeds to modeling. The goal is to minimize exchanges by ensuring every question is conditional on the previous answer, preventing irrelevant numbers or subjective advice.
+【改写前】
+- The consultation operates on a principle of 'mechanism-constraint-parameter' sequencing, with a strict prohibition against 'coaching-style' or 'prescriptive' questioning. The agent must treat the expert as a source of system dynamics and operational limits, not as a strategy consultant. The hierarchy is: first, establish the dominant behavioral mechanism; second, identify the primary operational constraint that limits that mechanism; third, calibrate the quantitative parameters within those constraints. Asking for a number before the behavior and its constraints are understood is a fatal error. Furthermore, asking for advice, recommendations, or 'what to do' is a prohibited category that wastes exchanges and introduces subjective bias not grounded in system physics.
+- If the agent has not yet established the dominant behavioral mechanism or the primary causal driver of the system's dynamics, the agent asks for the standard operational norm or the most common real-world pattern that defines how the system actually functions. This branch takes absolute priority. The condition is that the problem statement allows for multiple plausible physical or logical interpretations of the core process. The agent must not assume a generic theoretical ideal; it must ask for the prevailing practice in the specific context described. This branch resolves the 'shape' of the model. If two structural ambiguities exist, the agent asks about the one that determines the primary state transition or the main feedback loop.
+- Else, if the dominant behavioral mechanism has been established, but the agent has not yet identified the primary operational constraint or hard limit that governs the effectiveness of that mechanism, the agent asks for the specific constraint that limits the mechanism's application. This branch is critical because a mechanism without its limiting constraint leads to models that assume infinite or unbounded capability. The condition is that the agent knows *how* the system acts but does not know *what stops it* or *what it must not violate* to remain valid. The question must reference the established mechanism and ask for the specific boundary or trade-off that operators must navigate. For example, if the expert established that 'increasing outflow' is the primary lever, the agent must ask what limits that outflow before asking for the magnitude.
+- Else, if the dominant behavioral mechanism and its primary operational constraints have been established, but the model requires a specific quantitative parameter (such as a rate, threshold, duration, or proportion) that is critical to the dynamics and absent from the dataset, the agent asks for the typical empirical range or central estimate for that parameter. This branch applies only when the structural logic and its constraints are fixed. The condition is that the agent knows *how* the variable acts and *what limits it*, but does not know *how much* it acts. The question must explicitly reference the previously established mechanism and constraint to ensure the expert calibrates the value to that specific context, rather than providing </t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>The previous proposal was rejected for reproducing the parent policy. This patch rewrites the 'Interaction Strategy' section to explicitly enforce the 'mechanism-constraint-parameter' hierarchy and the prohibition on prescriptive questioning, which are key differentiators from the 'structural anchoring' and 'constraint-prioritization' policies in the evolution history that failed or were less effective. It ensures the agent asks for constraints before parameters, which addresses the 'modeling_rigorousness' and 'practicality' scores in the training evidence where models often lacked proper boundary conditions or relied on arbitrary parameters.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2003_C, 2017_D, 2024_C</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0.621652380753012</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>0.6181441846090282</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>-0.003508196143983788</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="n">
+        <v>4053</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>The consultation stops when its exchange budget is used: ten exchanges, one question each, as the policy's Interaction Limits section states. The policy states no other stop rule.</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t># Human Expert Interaction
+## Interaction Strategy
+The consultation operates on a 'mechanism-constraint-parameter' sequence, strictly prohibiting prescriptive or 'coaching-style' questions. The agent treats the expert as a source of system dynamics and operational limits, not a strategy advisor. The hierarchy is: establish the dominant behavioral mechanism, identify the primary operational constraint, then calibrate quantitative parameters. Asking for a number before understanding the behavior and its limits is a fatal error. Asking for advice or 'what to do' is prohibited.
+If the agent has not established the dominant behavioral mechanism or the primary causal driver, it asks for the standard operational norm or the most common real-world pattern defining how the system functions. This branch has absolute priority when the problem statement allows multiple plausible physical or logical interpretations of the core process. The agent must not assume a generic theoretical ideal; it must ask for the prevailing practice in the specific context. If two structural ambiguities exist, the agent asks about the one determining the primary state transition or main feedback loop.
+Else, if the dominant mechanism is established but the primary operational constraint or hard limit is not, the agent asks for the specific constraint limiting the mechanism's application. This branch is critical because a mechanism without its limiting constraint leads to models assuming infinite capability. The condition is that the agent knows *how* the system acts but not *what stops it* or *what it must not violate*. The question must reference the established mechanism and ask for the specific boundary or trade-off operators must navigate.
+Else, if the mechanism and its primary constraints are established, but the model requires a specific quantitative parameter (rate, threshold, duration, proportion) critical to dynamics and absent from the dataset, the agent asks for the typical empirical range or central estimate. This branch applies only when structural logic and constraints are fixed. The condition is that the agent knows *how* the variable acts and *what limits it*, but not *how much* it acts. The question must explicitly reference the previously established mechanism and constraint to ensure the expert calibrates the value to that specific context, not a generic textbook average. If tempted to ask for 'advice,' the agent must reframe the question into a parameter of the system's response dynamics.
+If none of the above conditions hold, or if the agent has gathered sufficient empirical grounding for the dominant mechanism, its constraints, and critical parameters, the agent stops asking and proceeds to modeling. The goal is to minimize exchanges by ensuring every question is conditional on the previous answer, preventing irrelevant numbers or subjective advice.
+Example interaction: The agent is modeling a competitive dynamic system. It first asks: 'Is the primary driver of state change a direct interaction between entities, or an indirect effect through a shared resource?' (Structural branch). Once the expert confirms it is a direct interaction, the agent asks: 'What is the primary constraint that limits the intensity of this interaction, such as a physical capacity or a regulatory limit?' (Constraint branch). Only after the expert identifies the limit, the agent asks: 'What is the typical magnitude of the interaction effect under these constraints?' (Parameter branch). It does not ask for 'strategic recommendations' or 'how to win,' because those are prescriptive and not system parameters.
+## Prohibited Requests
+The agent must not request feedback for:
+- coding, debugging, or implementation issues;
+- standard mathematical derivations;
+- computation or data processing.
+# Interaction Limits
+The consultation runs ten exchanges, one question each.
+After this policy terminates, the agent must not request further expert feedback for execution, computation, implementation, checking, or validation.</t>
+        </is>
+      </c>
+      <c r="V12" s="3" t="inlineStr">
+        <is>
+          <t>1. [agent_step] apply_policy_trigger
+Apply the complete natural-language interaction policy below to decide whether and when strategic expert feedback is required.
+# Human Expert Interaction
+## Interaction Strategy
+The consultation operates on a 'mechanism-constraint-parameter' sequence, strictly prohibiting prescriptive or 'coaching-style' questions. The agent treats the expert as a source of system dynamics and operational limits, not a strategy advisor. The hierarchy is: establish the dominant behavioral mechanism, identify the primary operational constraint, then calibrate quantitative parameters. Asking for a number before understanding the behavior and its limits is a fatal error. Asking for advice or 'what to do' is prohibited.
+If the agent has not established the dominant behavioral mechanism or the primary causal driver, it asks for the standard operational norm or the most common real-world pattern defining how the system functions. This branch has absolute priority when the problem statement allows multiple plausible physical or logical interpretations of the core process. The agent must not assume a generic theoretical ideal; it must ask for the prevailing practice in the specific context. If two structural ambiguities exist, the agent asks about the one determining the primary state transition or main feedback loop.
+Else, if the dominant mechanism is established but the primary operational constraint or hard limit is not, the agent asks for the specific constraint limiting the mechanism's application. This branch is critical because a mechanism without its limiting constraint leads to models assuming infinite capability. The condition is that the agent knows *how* the system acts but not *what stops it* or *what it must not violate*. The question must reference the established mechanism and ask for the specific boundary or trade-off operators must navigate.
+Else, if the mechanism and its primary constraints are established, but the model requires a specific quantitative parameter (rate, threshold, duration, proportion) critical to dynamics and absent from the dataset, the agent asks for the typical empirical range or central estimate. This branch applies only when structural logic and constraints are fixed. The condition is that the agent knows *how* the variable acts and *what limits it*, but not *how much* it acts. The question must explicitly reference the previously established mechanism and constraint to ensure the expert calibrates the value to that specific context, not a generic textbook average. If tempted to ask for 'advice,' the agent must reframe the question into a parameter of the system's response dynamics.
+If none of the above conditions hold, or if the agent has gathered sufficient empirical grounding for the dominant mechanism, its constraints, and critical parameters, the agent stops asking and proceeds to modeling. The goal is to minimize exchanges by ensuring every question is conditional on the previous answer, preventing irrelevant numbers or subjective advice.
+Example interaction: The agent is modeling a competitive dynamic system. It first asks: 'Is the primary driver of state change a direct interaction between entities, or an indirect effect through a shared resource?' (Structural branch). Once the expert confirms it is a direct interaction, the agent asks: 'What is the primary constraint that limits the intensity of this interaction, such as a physical capacity or a regulatory limit?' (Constraint branch). Only after the expert identifies the limit, the agent asks: 'What is the typical magnitude of the interaction effect under these constraints?' (Parameter branch). It does not ask for 'strategic recommendations' or 'how to win,' because those are prescriptive and not system parameters.
+## Prohibited Requests
+The agent must not request feedback for:
+- coding, debugging, or implementation issues;
+- standard mathematical derivations;
+- computation or data processing.
+# Interaction Limits
+The consultation runs ten exchanges, one question each.
+After this policy terminates, the agent must not request further expert feedback for execution, computation, implementation, checking, or validation.
+2. [expert_exchange] request_strategic_feedback
+When the interaction policy requires consultation, present the specified strategic context and request only the qualitative expert judgment defined by that policy.
+3. [agent_analysis] integrate_strategic_feedback
+Evaluate and apply the expert reply according to the interaction policy, then continue all technical modeling work autonomously.
+4. [close] close_policy_interaction
+Stop expert interaction at the stated limit or termination condition and complete the remaining modeling work autonomously.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V11"/>
+  <autoFilter ref="A1:V12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1985,7 +2125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:Q61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12650,8 +12790,1078 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Mechanism-Constraint-Parameter with Anti-Prescriptive Guard</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>interaction_workflow_c83b67c63c37</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>2003_C</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G56" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>In practice, about how many checked bags does each passenger at a large U.S. airport carry?</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>Q1: In practice, about how many checked bags does each passenger at a large U.S. airport carry?
+Q2: With ~1.2 bags per passenger, how long do passengers typically wait in the checked-bag drop line at a busy large airport?
+Q3: With screening lanes added at bag drop, how many minutes before departure do passengers generally need at minimum to avoid missing their flight?
+Q4: For the peak hour at a large airport, what share of the hour's flight departures is concentrated in the busiest 15 minutes?
+Q5: When an EDS machine breaks down, how is its screening load typically handled?
+Q6: In practice, how many EDS units do large airports typically keep as spare capacity so one breakdown doesn't stop screening?
+Q7: When a passenger with checked bags is delayed, what is the typical cost airlines prefer to avoid?
+Q8: How many days of screening demand do large airports typically hold checked bags for before they must be cleared?
+Q9: In the EDS vs ETD debate, what do airport security operators say is the main practical advantage of ETD?
+Q10: Besides peak hour, when else in the day do airports most often face bag-drop surges that strain screening capacity?</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>A1: About 1.0–1.3 checked bags per passenger on average at a large U.S. airport, with roughly 0.8–1.0 for domestic leisure travel and higher (1.3–1.6) on long-haul international routes. A common planning figure is about 1.2 checked bags per passenger. This is an empirical judgment, not a precise value.
+A2: At a busy large airport, checked-bag drop-line waits are typically about 10–20 minutes at peak, often 5–10 minutes off-peak, with occasional 30+ minute waits during holiday or disruption surges. These are empirical judgments, not precise values.
+A3: For a large U.S. airport with checked-bag screening at drop, passengers generally need to be at the bag-drop/screening lane roughly 45–60 minutes before departure to reliably avoid missing the flight. That reflects the combined bag-drop wait, screening time, and the airline's checked-bag cutoff (commonly 45 minutes domestic, 60 minutes international). A bare minimum of about 30–45 minutes is possible off-peak, but it is risky. This is an empirical judgment, not a precise value.
+A4: At a large U.S. airport, the busiest 15 minutes of a peak hour typically carries roughly 30–40% of that hour's departures, versus a uniform 25%. In strongly banked/hub operations it can reach about 40–45%. This is an empirical judgment, not a precise value.
+A5: When an EDS breaks down, its load is normally absorbed by the remaining operational EDS units at that airport, which run at their higher throughput (up to ~210 bags/hr) and take on the overflow; bags may be queued briefly until capacity frees up. If redundancy is insufficient, the fallback is manual/alternative screening — hand search or ETD — rather than leaving bags unscreened, since 100% screening is mandated. In practice airports size EDS counts with some spare capacity precisely so a single failure does not force a shutdown of the lane. This is an operational judgment, not a precise figure.
+A6: Large airports typically size EDS counts so that one unit's worth of capacity is spare — i.e., they deploy roughly one extra unit beyond the number needed to meet peak demand, giving N+1 redundancy. In practice this means about 10–15% spare capacity above the peak-hour requirement, which for a large airport usually works out to one, occasionally two, spare units. This is an operational judgment, not a precise figure.
+A7: Airlines' dominant cost from a delayed checked-bag passenger is the **misconnect/downstream disruption cost**, not the passenger's own inconvenience. In practice the airline prefers to avoid:
+- **A missed flight / misconnect**: rebooking, reaccommodation, and possible compensation — commonly on the order of a few hundred dollars per affected passenger (roughly $200–$500 domestic, higher for international), plus knock-on crew and gate costs.
+- **A delayed departure**: holding a flight for late bags/passengers propagates delay through the day's rotations, costing roughly tens to low hundreds of dollars per minute of block delay at the aircraft level.
+- **Bag-handling failures**: lost/delayed baggage claims, typically ~$100–$300 per mishandled bag in direct cost.
+So the cost they most want to avoid is the **misconnect and its downstream network delay**, which is generally far larger than the bag-drop wait itself. These are empirical judgments, not precise figures.
+A8: Large airports do not hold checked bags for days awaiting screening. Under the 100% screening mandate, every checked bag must be screened before it is loaded onto its flight — effectively same-day, within the departure window (typically cleared within the 1–2 hours before departure). There is no multi-day backlog of unscreened bags; bags are not stored awaiting clearance. So the practical "hold" horizon is hours, not days. This is an operational judgment, not a precise figure.
+A9: The main practical advantage operators cite for ETD is **flexibility and low space/labor footprint at the point of use** — it is a small, relatively inexpensive ($45k vs ~$1M) portable unit that can be deployed at gates, transfer points, and secondary-screening locations where an eight-ton EDS cannot physically go, and it can be brought to the bag rather than the bag to the machine.
+Secondarily, operators value ETD's **higher detection accuracy (99.7% vs 98.5%) and reliability (98% vs 92%)** as a confirmatory/secondary layer on top of EDS, which is why it is used for the higher-risk subset rather than as a primary bulk screener.
+Its practical disadvantage — much lower throughput (40–50 vs 160–210 bags/hr) and ~10× the labor cost per bag — is why operators treat it as a complement to EDS, not a replacement. This is an operational judgment, not a precise figure.
+A10: Besides the peak hour, the main bag-drop surges that strain screening capacity are:
+- **Early-morning departure bank** (roughly 05:00–08:00): the day's first wave of departures, when many business travelers and connecting banks push bags through in a short window; often the single busiest screening period at hub airports.
+- **Late-afternoon/early-evening departure bank** (roughly 16:00–19:00): the second major bank, driven by returning business travelers and international departures.
+- **Holiday and weekend peaks**: Thanksgiving, Christmas/New Year, and summer weekends produce surges well above normal daily peaks.
+- **Disruption surges**: weather, ATC, or a cancellation wave causes rebooked passengers to re-drop bags in concentrated bursts, plus the 2% daily cancellations reshuffling loads.
+These are empirical judgments, not precise figures.</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Human Expert Dialogue
+## Exchange 1
+**Modeling Agent question**
+In practice, about how many checked bags does each passenger at a large U.S. airport carry?
+**Human expert response**
+About 1.0–1.3 checked bags per passenger on average at a large U.S. airport, with roughly 0.8–1.0 for domestic leisure travel and higher (1.3–1.6) on long-haul international routes. A common planning figure is about 1.2 checked bags per passenger. This is an empirical judgment, not a precise value.
+## Exchange 2
+**Modeling Agent question**
+With ~1.2 bags per passenger, how long do passengers typically wait in the checked-bag drop line at a busy large airport?
+**Human expert response**
+At a busy large airport, checked-bag drop-line waits are typically about 10–20 minutes at peak, often 5–10 minutes off-peak, with occasional 30+ minute waits during holiday or disruption surges. These are empirical judgments, not precise values.
+## Exchange 3
+**Modeling Agent question**
+With screening lanes added at bag drop, how many minutes before departure do passengers generally need at minimum to avoid missing their flight?
+**Human expert response**
+For a large U.S. airport with checked-bag screening at drop, passengers generally need to be at the bag-drop/screening lane roughly 45–60 minutes before departure to reliably avoid missing the flight. That reflects the combined bag-drop wait, screening time, and the airline's checked-bag cutoff (commonly 45 minutes domestic, 60 minutes international). A bare minimum of about 30–45 minutes is possible off-peak, but it is risky. This is an empirical judgment, not a precise value.
+## Exchange 4
+**Modeling Agent question**
+For the peak hour at a large airport, what share of the hour's flight departures is concentrated in the busiest 15 minutes?
+**Human expert response**
+At a large U.S. airport, the busiest 15 minutes of a peak hour typically carries roughly 30–40% of that hour's departures, versus a uniform 25%. In strongly banked/hub operations it can reach about 40–45%. This is an empirical judgment, not a precise value.
+## Exchange 5
+**Modeling Agent question**
+When an EDS machine breaks down, how is its screening load typically handled?
+**Human expert response**
+When an EDS breaks down, its load is normally absorbed by the remaining operational EDS units at that airport, which run at their higher throughput (up to ~210 bags/hr) and take on the overflow; bags may be queued briefly until capacity frees up. If redundancy is insufficient, the fallback is manual/alternative screening — hand search or ETD — rather than leaving bags unscreened, since 100% screening is mandated. In practice airports size EDS counts with some spare capacity precisely so a single failure does not force a shutdown of the lane. This is an operational judgment, not a precise figure.
+## Exchange 6
+**Modeling Agent question**
+In practice, how many EDS units do large airports typically keep as spare capacity so one breakdown doesn't stop screening?
+**Human expert response**
+Large airports typically size EDS counts so that one unit's worth of capacity is spare — i.e., they deploy roughly one extra unit beyond the number needed to meet peak demand, giving N+1 redundancy. In practice this means about 10–15% spare capacity above the peak-hour requirement, which for a large airport usually works out to one, occasionally two, spare units. This is an operational judgment, not a precise figure.
+## Exchange 7
+**Modeling Agent question**
+When a passenger with checked bags is delayed, what is the typical cost airlines prefer to avoid?
+**Human expert response**
+Airlines' dominant cost from a delayed checked-bag passenger is the **misconnect/downstream disruption cost**, not the passenger's own inconvenience. In practice the airline prefers to avoid:
+- **A missed flight / misconnect**: rebooking, reaccommodation, and possible compensation — commonly on the order of a few hundred dollars per affected passenger (roughly $200–$500 domestic, higher for international), plus knock-on crew and gate costs.
+- **A delayed departure**: holding a flight for late bags/passengers propagates delay through the day's rotations, costing roughly tens to low hundreds of dollars per minute of block delay at the aircraft level.
+- **Bag-handling failures**: lost/delayed baggage claims, typically ~$100–$300 per mishandled bag in direct cost.
+So the cost they most want to avoid is the **misconnect and its downstream network delay**, which is generally far larger than the bag-drop wait itself. These are empirical judgments, not precise figures.
+## Exchange 8
+**Modeling Agent question**
+How many days of screening demand do large airports typically hold checked bags for before they must be cleared?
+**Human expert response**
+Large airports do not hold checked bags for days awaiting screening. Under the 100% screening mandate, every checked bag must be screened before it is loaded onto its flight — effectively same-day, within the departure window (typically cleared within the 1–2 hours before departure). There is no multi-day backlog of unscreened bags; bags are not stored awaiting clearance. So the practical "hold" horizon is hours, not days. This is an operational judgment, not a precise figure.
+## Exchange 9
+**Modeling Agent question**
+In the EDS vs ETD debate, what do airport security operators say is the main practical advantage of ETD?
+**Human expert response**
+The main practical advantage operators cite for ETD is **flexibility and low space/labor footprint at the point of use** — it is a small, relatively inexpensive ($45k vs ~$1M) portable unit that can be deployed at gates, transfer points, and secondary-screening locations where an eight-ton EDS cannot physically go, and it can be brought to the bag rather than the bag to the machine.
+Secondarily, operators value ETD's **higher detection accuracy (99.7% vs 98.5%) and reliability (98% vs 92%)** as a confirmatory/secondary layer on top of EDS, which is why it is used for the higher-risk subset rather than as a primary bulk screener.
+Its practical disadvantage — much lower throughput (40–50 vs 160–210 bags/hr) and ~10× the labor cost per bag — is why operators treat it as a complement to EDS, not a replacement. This is an operational judgment, not a precise figure.
+## Exchange 10
+**Modeling Agent question**
+Besides peak hour, when else in the day do airports most often face bag-drop surges that strain screening capacity?
+**Human expert response**
+Besides the peak hour, the main bag-drop surges that strain screening capacity are:
+- **Early-morning departure bank** (roughly 05:00–08:00): the day's first wave of departures, when many business travelers and connecting banks push bags through in a short window; often the single busiest screening period at hub airports.
+- **Late-afternoon/early-evening departure bank** (roughly 16:00–19:00): the second major bank, driven by returning business travelers and international departures.
+- **Holiday and weekend peaks**: Thanksgiving, Christmas/New Year, and summer weekends produce surges well above normal daily peaks.
+- **Disruption surges**: weather, ATC, or a cancellation wave causes rebooked passengers to re-drop bags in concentrated bursts, plus the 2% daily cancellations reshuffling loads.
+These are empirical judgments, not precise figures.
+</t>
+        </is>
+      </c>
+      <c r="L56" s="5" t="n">
+        <v>1675</v>
+      </c>
+      <c r="M56" s="6" t="n">
+        <v>12.85</v>
+      </c>
+      <c r="N56" s="4" t="n">
+        <v>0.6125</v>
+      </c>
+      <c r="O56" s="4" t="n">
+        <v>0.5738759872886825</v>
+      </c>
+      <c r="P56" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r1p1_20261003_160723</t>
+        </is>
+      </c>
+      <c r="Q56" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r1p1_20261003_160723/output/results/solution_report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Mechanism-Constraint-Parameter with Anti-Prescriptive Guard</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>interaction_workflow_c83b67c63c37</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>2003_C</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F57" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G57" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>When a large flight's checked bags arrive together at the security screening line during the busy hour, how do the operators actually handle them — all bags in one batch through the scanners, or one a…</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Q1: When a large flight's checked bags arrive together at the security screening line during the busy hour, how do the operators actually handle them — all bags in one batch through the scanners, or one at a time?
+Q2: What is the single hardest limit operators face when the scanner is the only screening step that must be finished before a plane departs?
+Q3: Given that a plane cannot leave until its last bag has finished scanning, how many minutes before the scheduled departure must a flight's bags start going through the scanners on a normal day?
+Q4: How many of the passengers on a full flight usually have at least one checked bag, as a typical share?
+Q5: When several flights have bags queuing for the same scanners at once, which flight's bags get scanned first in practice?
+Q6: How many minutes early do airlines normally get a flight's bags to the screening line, to leave slack if the scanners are busy?
+Q7: When scanners run more than one shift in a day, does the screening line stay open around the clock, or only during certain hours?
+Q8: If the scanners clear a bag but officers still suspect something, how common is a second manual re-check, and what usually triggers it?
+Q9: When a scanned bag is flagged, can it be manually re-checked right there in the screening area without stopping the whole line?
+Q10: During the busiest departure hour, is one screening line usually enough, or do the big airports spread the bags over several parallel lanes?</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>A1: In real EDS/ETD screening lines, bags are handled **one at a time through the scanner**, not as a single batch. Each bag is individually loaded onto the EDS belt (or fed to the ETD), scanned, and cleared or flagged before the next bag proceeds. A large flight's bags arrive as a stream and are queued, but the machine processes them serially at its rated throughput (160–210 bags/hr for EDS; 40–50 for ETD).
+The only "batching" that occurs is upstream: bags from one flight may be grouped or segregated by flight for reconciliation and to keep a flight's bags together, and cleared bags are consolidated for transport to the aircraft. But the scanning operation itself is strictly one bag per scan cycle. This is why capacity is modeled as a serial service rate, and why a large flight's bag volume translates into a queueing delay rather than a single bulk pass.
+A2: The hardest limit is the **serial service rate of the scanner itself** — the machine can only clear one bag per scan cycle, so the total bags from a flight must pass through a single-server bottleneck at 160–210 bags/hr (EDS). No amount of staffing or batching can make the scanner clear bags faster than that rate, so the departure cannot occur until the last bag of that flight has completed its scan.
+A3: There is no single fixed number — it depends on the flight's bag volume and the scanner's rate, so the required lead time is the time to clear the *last* bag of that flight.
+As an empirical rule of thumb: with EDS throughput of 160–210 bags/hr (roughly 2.7–3.5 bags/min), a flight's bags must begin scanning about **1 minute per 3 bags** of checked luggage, plus a small buffer for queueing and the 8% downtime. For a typical narrow-body flight (~100–150 checked bags) that is roughly **30–50 minutes** before departure; a large wide-body (~300–400 bags) needs on the order of **1.5–2 hours**. These are order-of-magnitude judgments, not precise values, and assume the scanner is dedicated to that flight's bags.
+A4: Typically **about 60–70% of passengers on a full flight check at least one bag** — a common planning figure is roughly two-thirds. This varies by route and carrier: on leisure-heavy long-haul flights the share runs higher (70–80%), while on short business-oriented routes it can be lower (40–50%). For a rough model, using ~0.6–0.7 checked bags per passenger, or about one checked bag per passenger as an upper bound, is a reasonable empirical judgment rather than a precise value.
+A5: In practice, the queue is **not strictly first-come-first-served by bag arrival**. The dominant real-world rule is **priority by departure time**: bags for the flight departing soonest are pushed to the front, because the binding constraint is making each plane's departure slot. This is usually implemented as a deadline-driven (earliest-departure-first) discipline, with bags from a flight close to its departure jumping ahead of a later flight's bags.
+Two secondary factors override or modify that:
+- **Flight segregation/reconciliation**: bags are kept grouped by flight, so the line often processes one flight's stream to completion before switching, rather than interleaving individual bags from many flights.
+- **Risk/priority flags**: higher-risk flights or those under secondary screening (EDS+ETD) may be given precedence regardless of departure time.
+So the practical ordering is earliest-departure-first, with flight-level batching and risk-based exceptions layered on top.
+A6: Airlines typically deliver a flight's checked bags to the screening line **about 45–60 minutes before scheduled departure** as a standard planning buffer, with wide-body/long-haul flights often starting **90–120 minutes** out. This is the industry norm for bag cut-off and screening lead time, not a precise figure.
+The slack is meant to absorb queueing behind other flights, the ~8% EDS downtime, and re-screening of flagged bags. It is a buffer over the pure scan time, not a fixed value — short-haul narrow-body flights may use as little as 30–40 minutes, while large international departures build in more. These are empirical judgments reflecting common airline practice.
+A7: Screening lines are **not run around the clock** at most airports. They operate in windows matched to the departure schedule — typically opening a few hours before the first wave of departures and closing after the last bank of the day clears, with the line idle overnight.
+Two qualifications:
+- **Hub airports with red-eye or international departures** may keep a screening line staffed through the night, but usually only a reduced subset of lanes, not the full complement.
+- **Staffing, not machine availability, is the binding constraint** on hours: EDS machines can run continuously, but the labor to operate them is scheduled in shifts, so the line's open hours track the flight banks rather than the clock.
+For a peak-hour model this matters only in that the peak-hour demand is what sizes the line; off-peak hours are handled with fewer active lanes.
+A8: A second manual re-check is **uncommon but routine** — on the order of a few percent of bags, not a large share. Most bags clear on the EDS image alone.
+Typical triggers:
+- **Operator-flagged anomalies**: the EDS image shows an unresolved dense mass, an odd shape, or an object the operator cannot classify, even though the automated alarm did not fire.
+- **Automated alarm requiring resolution**: when the EDS *does* alarm, the bag is not simply passed — it is pulled for manual inspection or ETD swab, which is the standard resolution step.
+- **Random or risk-based selection**: a small percentage of cleared bags are pulled for random secondary screening, and higher-risk flights/passengers get extra scrutiny.
+- **ETD confirmation**: under the dual-screening policy, flagged bags go to ETD for trace confirmation.
+So re-checks are driven mainly by operator judgment on ambiguous images and by alarm resolution, plus a small random/risk-based fraction. This is an empirical judgment, not a precise rate.
+A9: Yes. A flagged bag is pulled off the main line to a separate inspection position (a secondary/resolution table or an ETD station) and resolved there by hand, while the scanner keeps processing the remaining bags. The line does not stop.
+The only conditions under which it would slow or stop the line: if the resolution area is unstaffed or already occupied, the flagged bag may sit and briefly block the offload end; and if a bag alarms and cannot be cleared, it may trigger a broader hold on that flight's bags. But routine manual re-checks are handled in parallel with scanning, not by halting the belt.
+A10: At large airports, bags are spread over **several parallel lanes**, not one. A single EDS lane at 160–210 bags/hr cannot absorb a peak-hour wave from multiple large flights — the combined bag volume would exceed one machine's serial rate and blow past departure deadlines. So the peak hour is served by a bank of parallel lanes (commonly several to a dozen or more at a major hub), each an independent EDS line, with bags assigned across them.
+Two qualifications:
+- **Lanes are pooled, not dedicated per flight**: any flight's bags can feed any open lane, and the earliest-departure-first discipline is applied across the whole bank.
+- **The number of active lanes scales with the peak**, not the daily average — off-peak hours run fewer lanes.
+So for a peak-hour model, the relevant quantity is the *number of parallel lanes* needed to clear the peak bag volume in time, not whether one line suffices. This is an empirical judgment reflecting hub practice.</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Human Expert Dialogue
+## Exchange 1
+**Modeling Agent question**
+When a large flight's checked bags arrive together at the security screening line during the busy hour, how do the operators actually handle them — all bags in one batch through the scanners, or one at a time?
+**Human expert response**
+In real EDS/ETD screening lines, bags are handled **one at a time through the scanner**, not as a single batch. Each bag is individually loaded onto the EDS belt (or fed to the ETD), scanned, and cleared or flagged before the next bag proceeds. A large flight's bags arrive as a stream and are queued, but the machine processes them serially at its rated throughput (160–210 bags/hr for EDS; 40–50 for ETD).
+The only "batching" that occurs is upstream: bags from one flight may be grouped or segregated by flight for reconciliation and to keep a flight's bags together, and cleared bags are consolidated for transport to the aircraft. But the scanning operation itself is strictly one bag per scan cycle. This is why capacity is modeled as a serial service rate, and why a large flight's bag volume translates into a queueing delay rather than a single bulk pass.
+## Exchange 2
+**Modeling Agent question**
+What is the single hardest limit operators face when the scanner is the only screening step that must be finished before a plane departs?
+**Human expert response**
+The hardest limit is the **serial service rate of the scanner itself** — the machine can only clear one bag per scan cycle, so the total bags from a flight must pass through a single-server bottleneck at 160–210 bags/hr (EDS). No amount of staffing or batching can make the scanner clear bags faster than that rate, so the departure cannot occur until the last bag of that flight has completed its scan.
+## Exchange 3
+**Modeling Agent question**
+Given that a plane cannot leave until its last bag has finished scanning, how many minutes before the scheduled departure must a flight's bags start going through the scanners on a normal day?
+**Human expert response**
+There is no single fixed number — it depends on the flight's bag volume and the scanner's rate, so the required lead time is the time to clear the *last* bag of that flight.
+As an empirical rule of thumb: with EDS throughput of 160–210 bags/hr (roughly 2.7–3.5 bags/min), a flight's bags must begin scanning about **1 minute per 3 bags** of checked luggage, plus a small buffer for queueing and the 8% downtime. For a typical narrow-body flight (~100–150 checked bags) that is roughly **30–50 minutes** before departure; a large wide-body (~300–400 bags) needs on the order of **1.5–2 hours**. These are order-of-magnitude judgments, not precise values, and assume the scanner is dedicated to that flight's bags.
+## Exchange 4
+**Modeling Agent question**
+How many of the passengers on a full flight usually have at least one checked bag, as a typical share?
+**Human expert response**
+Typically **about 60–70% of passengers on a full flight check at least one bag** — a common planning figure is roughly two-thirds. This varies by route and carrier: on leisure-heavy long-haul flights the share runs higher (70–80%), while on short business-oriented routes it can be lower (40–50%). For a rough model, using ~0.6–0.7 checked bags per passenger, or about one checked bag per passenger as an upper bound, is a reasonable empirical judgment rather than a precise value.
+## Exchange 5
+**Modeling Agent question**
+When several flights have bags queuing for the same scanners at once, which flight's bags get scanned first in practice?
+**Human expert response**
+In practice, the queue is **not strictly first-come-first-served by bag arrival**. The dominant real-world rule is **priority by departure time**: bags for the flight departing soonest are pushed to the front, because the binding constraint is making each plane's departure slot. This is usually implemented as a deadline-driven (earliest-departure-first) discipline, with bags from a flight close to its departure jumping ahead of a later flight's bags.
+Two secondary factors override or modify that:
+- **Flight segregation/reconciliation**: bags are kept grouped by flight, so the line often processes one flight's stream to completion before switching, rather than interleaving individual bags from many flights.
+- **Risk/priority flags**: higher-risk flights or those under secondary screening (EDS+ETD) may be given precedence regardless of departure time.
+So the practical ordering is earliest-departure-first, with flight-level batching and risk-based exceptions layered on top.
+## Exchange 6
+**Modeling Agent question**
+How many minutes early do airlines normally get a flight's bags to the screening line, to leave slack if the scanners are busy?
+**Human expert response**
+Airlines typically deliver a flight's checked bags to the screening line **about 45–60 minutes before scheduled departure** as a standard planning buffer, with wide-body/long-haul flights often starting **90–120 minutes** out. This is the industry norm for bag cut-off and screening lead time, not a precise figure.
+The slack is meant to absorb queueing behind other flights, the ~8% EDS downtime, and re-screening of flagged bags. It is a buffer over the pure scan time, not a fixed value — short-haul narrow-body flights may use as little as 30–40 minutes, while large international departures build in more. These are empirical judgments reflecting common airline practice.
+## Exchange 7
+**Modeling Agent question**
+When scanners run more than one shift in a day, does the screening line stay open around the clock, or only during certain hours?
+**Human expert response**
+Screening lines are **not run around the clock** at most airports. They operate in windows matched to the departure schedule — typically opening a few hours before the first wave of departures and closing after the last bank of the day clears, with the line idle overnight.
+Two qualifications:
+- **Hub airports with red-eye or international departures** may keep a screening line staffed through the night, but usually only a reduced subset of lanes, not the full complement.
+- **Staffing, not machine availability, is the binding constraint** on hours: EDS machines can run continuously, but the labor to operate them is scheduled in shifts, so the line's open hours track the flight banks rather than the clock.
+For a peak-hour model this matters only in that the peak-hour demand is what sizes the line; off-peak hours are handled with fewer active lanes.
+## Exchange 8
+**Modeling Agent question**
+If the scanners clear a bag but officers still suspect something, how common is a second manual re-check, and what usually triggers it?
+**Human expert response**
+A second manual re-check is **uncommon but routine** — on the order of a few percent of bags, not a large share. Most bags clear on the EDS image alone.
+Typical triggers:
+- **Operator-flagged anomalies**: the EDS image shows an unresolved dense mass, an odd shape, or an object the operator cannot classify, even though the automated alarm did not fire.
+- **Automated alarm requiring resolution**: when the EDS *does* alarm, the bag is not simply passed — it is pulled for manual inspection or ETD swab, which is the standard resolution step.
+- **Random or risk-based selection**: a small percentage of cleared bags are pulled for random secondary screening, and higher-risk flights/passengers get extra scrutiny.
+- **ETD confirmation**: under the dual-screening policy, flagged bags go to ETD for trace confirmation.
+So re-checks are driven mainly by operator judgment on ambiguous images and by alarm resolution, plus a small random/risk-based fraction. This is an empirical judgment, not a precise rate.
+## Exchange 9
+**Modeling Agent question**
+When a scanned bag is flagged, can it be manually re-checked right there in the screening area without stopping the whole line?
+**Human expert response**
+Yes. A flagged bag is pulled off the main line to a separate inspection position (a secondary/resolution table or an ETD station) and resolved there by hand, while the scanner keeps processing the remaining bags. The line does not stop.
+The only conditions under which it would slow or stop the line: if the resolution area is unstaffed or already occupied, the flagged bag may sit and briefly block the offload end; and if a bag alarms and cannot be cleared, it may trigger a broader hold on that flight's bags. But routine manual re-checks are handled in parallel with scanning, not by halting the belt.
+## Exchange 10
+**Modeling Agent question**
+During the busiest departure hour, is one screening line usually enough, or do the big airports spread the bags over several parallel lanes?
+**Human expert response**
+At large airports, bags are spread over **several parallel lanes**, not one. A single EDS lane at 160–210 bags/hr cannot absorb a peak-hour wave from multiple large flights — the combined bag volume would exceed one machine's serial rate and blow past departure deadlines. So the peak hour is served by a bank of parallel lanes (commonly several to a dozen or more at a major hub), each an independent EDS line, with bags assigned across them.
+Two qualifications:
+- **Lanes are pooled, not dedicated per flight**: any flight's bags can feed any open lane, and the earliest-departure-first discipline is applied across the whole bank.
+- **The number of active lanes scales with the peak**, not the daily average — off-peak hours run fewer lanes.
+So for a peak-hour model, the relevant quantity is the *number of parallel lanes* needed to clear the peak bag volume in time, not whether one line suffices. This is an empirical judgment reflecting hub practice.
+</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="n">
+        <v>2272</v>
+      </c>
+      <c r="M57" s="6" t="n">
+        <v>17.69</v>
+      </c>
+      <c r="N57" s="4" t="n">
+        <v>0.6208333333333333</v>
+      </c>
+      <c r="O57" s="4" t="n">
+        <v>0.5738759872886825</v>
+      </c>
+      <c r="P57" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r2p1_20261003_160723</t>
+        </is>
+      </c>
+      <c r="Q57" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r2p1_20261003_160723/output/results/solution_report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Mechanism-Constraint-Parameter with Anti-Prescriptive Guard</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>interaction_workflow_c83b67c63c37</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>2017_D</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G58" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>At a busy airport security checkpoint, which single step causes passengers to wait longest and pile up most: the ID-check counter, the X-ray belt, or the millimeter-wave body scanner?</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Q1: At a busy airport security checkpoint, which single step causes passengers to wait longest and pile up most: the ID-check counter, the X-ray belt, or the millimeter-wave body scanner?
+Q2: You said the X-ray belt is the main bottleneck because bags pass one at a time through the machine and an officer reviews the image. What stops a single X-ray belt from processing bags much faster — is it the belt's physical speed, the officer reviewing images, or something else?
+Q3: You said the officer's decision on each bag's X-ray image is what caps the belt. For a normal, unflagged bag, roughly how many seconds does that officer take per image on average?
+Q4: At a typical US airport checkpoint on a normal day, what fraction of bags get flagged for a secondary hand search by the officer — roughly what percent?
+Q5: When a passenger walks through the millimeter-wave body scanner, what fraction get stopped for a pat-down by an officer, on a normal day?
+Q6: At a regular (non-Pre-Check) lane, how long does a passenger typically take to remove shoes, jacket, belt, electronics and liquids into bins, then put everything back after the scan?
+Q7: You said divesting is faster for experienced travelers and slower for families or infrequent flyers. How much slower, roughly, does a first-time or family traveler take to divest compared to a frequent flyer?
+Q8: In a security queue, some cultures strictly hold their place in line while others are more willing to squeeze in or let a friend join ahead. How does that tendency to let people cut in affect the smoothness of a queue?
+Q9: The problem says about 45% of US passengers enroll in Pre-Check, but only one Pre-Check lane is open for every three regular lanes. On a normal busy day, is the Pre-Check line usually shorter or longer than a regular line?
+Q10: At the first ID-check counter where an officer verifies a passenger's ID and boarding pass, how long does one officer typically spend per passenger on a busy day?</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>A1: The X-ray belt is the dominant bottleneck.
+Reason: it is the only step where every passenger's throughput is gated by a shared, serial resource — the conveyor and the single X-ray image reviewer — and where each passenger's service time is inflated by divesting and reclaiming multiple bins (shoes, jackets, electronics, liquids, laptops). Divesting/reclaiming alone typically takes tens of seconds per passenger, and flagged bags add unpredictable extra service. ID check is fast (a few seconds per passenger) and easily parallelized by adding officers; the body scanner is also short (a few seconds) and parallelizable by adding lanes. The X-ray belt, by contrast, has a hard mechanical throughput ceiling and long, variable per-passenger occupancy, so queues and variance concentrate there.
+This is an empirical judgment based on typical checkpoint service times, not a computed result.
+A2: The binding constraint is usually the human image reviewer, not the belt's physical speed.
+The belt itself moves at a fixed, modest speed (roughly 0.2–0.3 m/s), but that only sets a floor on spacing between bags. The real limit is that each bag's image must be visually interpreted by a screening officer, who must decide clear/flag, and who can only attend to one image stream at a time. That decision time — a few seconds per bag, longer for cluttered or flagged bags — is what caps throughput, and it is why one belt cannot simply be sped up to process more bags.
+Secondary factors: bags must be spaced so images don't overlap, and divesting/reclaiming at the belt ends creates gaps and surges. But if you removed the reviewer constraint, the belt speed and spacing alone would allow considerably higher throughput.
+This is an empirical judgment, not a computed result.
+A3: Roughly 3–6 seconds per normal, unflagged bag image — an empirical judgment, not a measured figure.
+That covers the officer's glance, pattern recognition, and clear/flag decision, plus the small handling gap between consecutive images. It is the same order as the belt's own spacing floor, which is why the reviewer, not belt speed, sets the ceiling. Cluttered or flagged bags take noticeably longer (often 10–30+ seconds once a secondary search is involved), which is what drives the variance.
+A4: Roughly 5–15% of bags get flagged for secondary hand search on a normal day — an empirical judgment, not a measured figure.
+Most bags clear on the image alone; flags come from cluttered/overlapping images, ambiguous items, and random or alarm-triggered selections. The rate rises with passenger volume, bag clutter, and tightened security posture, and can spike well above this range on high-alert days.
+A5: Roughly 2–5% of passengers get stopped for a pat-down on a normal day — an empirical judgment, not a measured figure.
+Most passengers clear the scanner or metal detector on the first pass. Pat-downs are triggered by alarms (metal, anomalies), random selection, and opt-outs, and the rate rises with tightened security posture or higher alarm sensitivity.
+A6: Roughly 30–60 seconds total for a typical regular-lane passenger — an empirical judgment, not a measured figure.
+That splits into two parts: divesting (removing shoes, belt, jacket, emptying pockets, pulling out laptop and liquids, loading bins) typically takes about 20–40 seconds, and reclaiming (collecting bins, re-dressing, repacking) about 10–20 seconds. It is faster for experienced travelers and slower for families, infrequent flyers, and those with many items. Pre-Check passengers skip shoes, belt, jacket, and laptop removal, cutting this to roughly half.
+A7: Roughly 2–3× slower — an empirical judgment, not a measured figure.
+A frequent flyer who knows the routine divests in about 15–25 seconds. A first-time or family traveler typically takes 45–90+ seconds, because of unfamiliarity with the rules, multiple people and bags to manage, children needing help, and repeated trips to the bin. Families with young children or groups with many items can exceed that, and the spread (variance) is much wider than the mean difference.
+A8: Letting people cut in degrades queue smoothness, mainly by breaking the first-come-first-served discipline that keeps a single-file queue orderly.
+Effects:
+- It adds unaccounted arrivals at the front, so the effective service rate seen by waiting passengers drops and their wait times rise unpredictably.
+- It creates local congestion and jostling at the merge point, which can physically slow the line and cause gaps upstream.
+- It increases variance: whether and when someone cuts is irregular, so wait times become less predictable even at constant throughput.
+- It can trigger defensive behavior (people crowding forward, guarding their spot), which further disrupts spacing and flow.
+The magnitude depends on how often it happens and whether it is tolerated by those behind. A culture that strictly holds place produces a smoother, more predictable queue; one that tolerates cutting produces a faster-moving but more erratic and less fair-feeling line. This is a qualitative judgment, not a measured result.
+A9: Pre-Check is usually shorter — often much shorter — despite the lane ratio.
+Reason: Pre-Check passengers move faster at every step (no shoe/belt/jacket/laptop removal, so divesting and reclaiming are roughly halved), so each open Pre-Check lane has both a higher service rate and a lower per-passenger service time. With 45% of passengers spread over one lane for every three regular lanes, the Pre-Check lane carries about 45/25 ≈ 1.8× the passenger volume of a regular lane, but its throughput per lane is also higher, so the queue is typically shorter and less variable.
+Caveat: this holds on normal days. Because there are so few Pre-Check lanes, a surge or a single slow/flagged passenger can make the Pre-Check line spike sharply, so its wait is shorter on average but can be less predictable. This is an empirical judgment, not a computed result.
+A10: Roughly 5–15 seconds per passenger on a busy day — an empirical judgment, not a measured figure.
+That covers the officer taking the ID and boarding pass, glancing at the photo and name, matching them to the passenger, and waving them through. It is fast and fairly consistent, which is why ID check rarely becomes the bottleneck: it is easily parallelized by opening more counters, and its service time is short and low-variance compared with divesting/reclaiming at the X-ray belt. Longer times occur mainly for flagged documents, secondary verification, or confused passengers, but those are a small minority.</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Human Expert Dialogue
+## Exchange 1
+**Modeling Agent question**
+At a busy airport security checkpoint, which single step causes passengers to wait longest and pile up most: the ID-check counter, the X-ray belt, or the millimeter-wave body scanner?
+**Human expert response**
+The X-ray belt is the dominant bottleneck.
+Reason: it is the only step where every passenger's throughput is gated by a shared, serial resource — the conveyor and the single X-ray image reviewer — and where each passenger's service time is inflated by divesting and reclaiming multiple bins (shoes, jackets, electronics, liquids, laptops). Divesting/reclaiming alone typically takes tens of seconds per passenger, and flagged bags add unpredictable extra service. ID check is fast (a few seconds per passenger) and easily parallelized by adding officers; the body scanner is also short (a few seconds) and parallelizable by adding lanes. The X-ray belt, by contrast, has a hard mechanical throughput ceiling and long, variable per-passenger occupancy, so queues and variance concentrate there.
+This is an empirical judgment based on typical checkpoint service times, not a computed result.
+## Exchange 2
+**Modeling Agent question**
+You said the X-ray belt is the main bottleneck because bags pass one at a time through the machine and an officer reviews the image. What stops a single X-ray belt from processing bags much faster — is it the belt's physical speed, the officer reviewing images, or something else?
+**Human expert response**
+The binding constraint is usually the human image reviewer, not the belt's physical speed.
+The belt itself moves at a fixed, modest speed (roughly 0.2–0.3 m/s), but that only sets a floor on spacing between bags. The real limit is that each bag's image must be visually interpreted by a screening officer, who must decide clear/flag, and who can only attend to one image stream at a time. That decision time — a few seconds per bag, longer for cluttered or flagged bags — is what caps throughput, and it is why one belt cannot simply be sped up to process more bags.
+Secondary factors: bags must be spaced so images don't overlap, and divesting/reclaiming at the belt ends creates gaps and surges. But if you removed the reviewer constraint, the belt speed and spacing alone would allow considerably higher throughput.
+This is an empirical judgment, not a computed result.
+## Exchange 3
+**Modeling Agent question**
+You said the officer's decision on each bag's X-ray image is what caps the belt. For a normal, unflagged bag, roughly how many seconds does that officer take per image on average?
+**Human expert response**
+Roughly 3–6 seconds per normal, unflagged bag image — an empirical judgment, not a measured figure.
+That covers the officer's glance, pattern recognition, and clear/flag decision, plus the small handling gap between consecutive images. It is the same order as the belt's own spacing floor, which is why the reviewer, not belt speed, sets the ceiling. Cluttered or flagged bags take noticeably longer (often 10–30+ seconds once a secondary search is involved), which is what drives the variance.
+## Exchange 4
+**Modeling Agent question**
+At a typical US airport checkpoint on a normal day, what fraction of bags get flagged for a secondary hand search by the officer — roughly what percent?
+**Human expert response**
+Roughly 5–15% of bags get flagged for secondary hand search on a normal day — an empirical judgment, not a measured figure.
+Most bags clear on the image alone; flags come from cluttered/overlapping images, ambiguous items, and random or alarm-triggered selections. The rate rises with passenger volume, bag clutter, and tightened security posture, and can spike well above this range on high-alert days.
+## Exchange 5
+**Modeling Agent question**
+When a passenger walks through the millimeter-wave body scanner, what fraction get stopped for a pat-down by an officer, on a normal day?
+**Human expert response**
+Roughly 2–5% of passengers get stopped for a pat-down on a normal day — an empirical judgment, not a measured figure.
+Most passengers clear the scanner or metal detector on the first pass. Pat-downs are triggered by alarms (metal, anomalies), random selection, and opt-outs, and the rate rises with tightened security posture or higher alarm sensitivity.
+## Exchange 6
+**Modeling Agent question**
+At a regular (non-Pre-Check) lane, how long does a passenger typically take to remove shoes, jacket, belt, electronics and liquids into bins, then put everything back after the scan?
+**Human expert response**
+Roughly 30–60 seconds total for a typical regular-lane passenger — an empirical judgment, not a measured figure.
+That splits into two parts: divesting (removing shoes, belt, jacket, emptying pockets, pulling out laptop and liquids, loading bins) typically takes about 20–40 seconds, and reclaiming (collecting bins, re-dressing, repacking) about 10–20 seconds. It is faster for experienced travelers and slower for families, infrequent flyers, and those with many items. Pre-Check passengers skip shoes, belt, jacket, and laptop removal, cutting this to roughly half.
+## Exchange 7
+**Modeling Agent question**
+You said divesting is faster for experienced travelers and slower for families or infrequent flyers. How much slower, roughly, does a first-time or family traveler take to divest compared to a frequent flyer?
+**Human expert response**
+Roughly 2–3× slower — an empirical judgment, not a measured figure.
+A frequent flyer who knows the routine divests in about 15–25 seconds. A first-time or family traveler typically takes 45–90+ seconds, because of unfamiliarity with the rules, multiple people and bags to manage, children needing help, and repeated trips to the bin. Families with young children or groups with many items can exceed that, and the spread (variance) is much wider than the mean difference.
+## Exchange 8
+**Modeling Agent question**
+In a security queue, some cultures strictly hold their place in line while others are more willing to squeeze in or let a friend join ahead. How does that tendency to let people cut in affect the smoothness of a queue?
+**Human expert response**
+Letting people cut in degrades queue smoothness, mainly by breaking the first-come-first-served discipline that keeps a single-file queue orderly.
+Effects:
+- It adds unaccounted arrivals at the front, so the effective service rate seen by waiting passengers drops and their wait times rise unpredictably.
+- It creates local congestion and jostling at the merge point, which can physically slow the line and cause gaps upstream.
+- It increases variance: whether and when someone cuts is irregular, so wait times become less predictable even at constant throughput.
+- It can trigger defensive behavior (people crowding forward, guarding their spot), which further disrupts spacing and flow.
+The magnitude depends on how often it happens and whether it is tolerated by those behind. A culture that strictly holds place produces a smoother, more predictable queue; one that tolerates cutting produces a faster-moving but more erratic and less fair-feeling line. This is a qualitative judgment, not a measured result.
+## Exchange 9
+**Modeling Agent question**
+The problem says about 45% of US passengers enroll in Pre-Check, but only one Pre-Check lane is open for every three regular lanes. On a normal busy day, is the Pre-Check line usually shorter or longer than a regular line?
+**Human expert response**
+Pre-Check is usually shorter — often much shorter — despite the lane ratio.
+Reason: Pre-Check passengers move faster at every step (no shoe/belt/jacket/laptop removal, so divesting and reclaiming are roughly halved), so each open Pre-Check lane has both a higher service rate and a lower per-passenger service time. With 45% of passengers spread over one lane for every three regular lanes, the Pre-Check lane carries about 45/25 ≈ 1.8× the passenger volume of a regular lane, but its throughput per lane is also higher, so the queue is typically shorter and less variable.
+Caveat: this holds on normal days. Because there are so few Pre-Check lanes, a surge or a single slow/flagged passenger can make the Pre-Check line spike sharply, so its wait is shorter on average but can be less predictable. This is an empirical judgment, not a computed result.
+## Exchange 10
+**Modeling Agent question**
+At the first ID-check counter where an officer verifies a passenger's ID and boarding pass, how long does one officer typically spend per passenger on a busy day?
+**Human expert response**
+Roughly 5–15 seconds per passenger on a busy day — an empirical judgment, not a measured figure.
+That covers the officer taking the ID and boarding pass, glancing at the photo and name, matching them to the passenger, and waving them through. It is fast and fairly consistent, which is why ID check rarely becomes the bottleneck: it is easily parallelized by opening more counters, and its service time is short and low-variance compared with divesting/reclaiming at the X-ray belt. Longer times occur mainly for flagged documents, secondary verification, or confused passengers, but those are a small minority.
+</t>
+        </is>
+      </c>
+      <c r="L58" s="5" t="n">
+        <v>2145</v>
+      </c>
+      <c r="M58" s="6" t="n">
+        <v>14.61</v>
+      </c>
+      <c r="N58" s="4" t="n">
+        <v>0.7125</v>
+      </c>
+      <c r="O58" s="4" t="n">
+        <v>0.6697362038348276</v>
+      </c>
+      <c r="P58" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r1p2_20261003_160723</t>
+        </is>
+      </c>
+      <c r="Q58" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r1p2_20261003_160723/output/results/solution_report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Mechanism-Constraint-Parameter with Anti-Prescriptive Guard</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>interaction_workflow_c83b67c63c37</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>2017_D</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F59" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G59" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Do passengers finish the body scan before they reach the belt to collect their bags?</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Q1: Do passengers finish the body scan before they reach the belt to collect their bags?
+Q2: On a busy morning, which step causes most of the piling up?
+Q3: Out of roughly 100 bags going through the X-ray, how many usually get flagged for a closer look?
+Q4: How many minutes does a closer manual inspection usually take?
+Q5: How many passengers, one after another, can one open lane screen per hour?
+Q6: How many passengers reach the checkpoint in a minute during a busy morning?
+Q7: Of all passengers using a checkpoint on a typical day, what share is in Pre-Check?
+Q8: When the line grows long, do most travelers switch to an open lane?
+Q9: Do people tend to bring more bags and bins into the screening lane?
+Q10: How long does checking one traveler's ID and boarding pass usually take?</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>A1: No — not necessarily, and in the described process the two are decoupled.
+The passenger's belongings go through the X-ray on the conveyor belt while the passenger separately goes through the millimeter wave scanner or metal detector. These are parallel streams, so a passenger can reach the post-X-ray belt to collect bags before, at roughly the same time as, or after finishing the body scan, depending on the relative service times of the two streams and any queueing at each.
+In practice the body scan (plus possible pat-down in Zone D) is often the longer or more variable step, so many passengers arrive at the belt and wait for their bags, but the reverse also occurs. The process does not enforce a fixed ordering between body-scan completion and belt arrival.
+A2: On a busy morning, the bottleneck is almost always the **X-ray/bag-screening stream and the downstream Zone D secondary screening**, not the ID check or the body scanner itself.
+Reasons: the X-ray conveyor is a single shared resource per lane with a long, variable service time (bins, laptops, liquids, flagged items), and any bag flagged for additional search pulls a security officer off the line, creating a compounding slowdown. Body scanning is comparatively fast and parallelizable across lanes. ID check is quick and rarely the constraint.
+So the piling up concentrates at the **queue feeding the X-ray lanes (Zone B) and at the post-X-ray belt**, where passengers wait for their belongings — with secondary screening (Zone D) as the main source of variance. This is an empirical judgment based on typical checkpoint behavior, not a precise measured value.
+A3: Roughly 5–15 out of 100 bags, i.e. on the order of 10%, is the usual flag rate for X-ray secondary screening at a US checkpoint. This is an empirical judgment, not a precise measured value; the rate varies with the mix of passengers, the items carried, and how aggressively the operator is set to flag. Pre-Check bags tend to be flagged at a lower rate than regular-lane bags.
+A4: Typically on the order of **1–3 minutes** for a routine manual bag inspection, with a central estimate around **2 minutes**. Simple re-scans or a quick swab are faster (under a minute); a full unpack-and-search, explosives-trace swab, or a pat-down can run **3–5 minutes or more**. The distribution is right-skewed, so a small fraction of inspections take much longer and drive most of the variance. This is an empirical judgment, not a precise measured value.
+A5: Roughly **100–200 passengers per hour per open lane**, with a central estimate around **150/hour** for a regular lane under normal conditions. This is an empirical judgment, not a precise measured value.
+The range reflects real-world variation: a well-staffed lane with few flagged bags and experienced passengers can approach 200/hour, while a lane slowed by heavy bin use, many laptops/liquids, frequent secondary screening, or Pre-Check-style mixed flow can drop toward 100/hour or below. Pre-Check lanes run higher (often 200–300/hour) because passengers divest less and are flagged less often.
+A6: Roughly **10–30 passengers per minute** arriving at a single checkpoint during a busy morning peak, with a central estimate around **15–20/minute**. This is an empirical judgment, not a precise measured value.
+The range reflects real-world variation: a large hub checkpoint at peak can approach 30/minute, while a smaller or moderately busy checkpoint runs nearer 10/minute. Note this is the *arrival* rate; it should be compared against lane capacity (roughly 150/hour per lane, i.e. ~2.5/minute per lane) to see how many lanes must be open to keep the queue stable.
+A7: Roughly **40–50%**, with a central estimate around **45%** — the problem statement itself cites about 45% enrollment in Pre-Check. This is an empirical judgment for a typical US checkpoint; the actual share varies by airport and time of day, and is often lower at smaller airports and higher at large hubs with many frequent/business travelers.
+A8: No — most travelers do not switch lanes when the line grows long.
+In a standard checkpoint, passengers commit to a lane once they enter the Zone B queue feeding a specific screening line; the physical layout (railings, single-file queue, belongings already on the belt) makes switching impractical or impossible. Travelers generally stay in their chosen lane and wait.
+Switching mainly happens at the earlier stage — when a passenger is choosing which lane to join — and even then most people pick the nearest or shortest-looking queue and stay. The social norm against "cutting" (noted in the problem) further discourages mid-queue lane changes. So a long line mostly lengthens waiting rather than redistributing passengers across open lanes. This is an empirical judgment, not a measured value.
+A9: Yes — most passengers bring multiple items into the lane, not just one bag.
+Typical travelers arrive with a carry-on plus a personal item (purse, backpack, laptop bag), and each of those plus the divested items (shoes, belt, jacket, electronics, liquids, laptop) goes into its own bin. So a single passenger commonly occupies **2–4 bins** on the belt, and a family or a heavy traveler can occupy considerably more.
+This matters because bin count, not passenger count, is what loads the X-ray conveyor: more bins per passenger means longer belt occupancy and slower effective throughput per lane. Pre-Check passengers use fewer bins (no shoe/belt/jacket removal, laptop stays in bag), which is a large part of why their lanes run faster. This is an empirical judgment, not a measured value.
+A10: Typically on the order of **10–20 seconds** per traveler for a routine ID and boarding-pass check, with a central estimate around **15 seconds**. This is an empirical judgment, not a precise measured value.
+The range reflects real-world variation: a quick glance-and-wave for a familiar or Pre-Check traveler can be under 10 seconds, while a slower check (document scrutiny, questions, a traveler fumbling for documents, or a flagged boarding pass) can run 30 seconds or more. It is one of the fastest steps in the checkpoint and rarely the bottleneck.</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Human Expert Dialogue
+## Exchange 1
+**Modeling Agent question**
+Do passengers finish the body scan before they reach the belt to collect their bags?
+**Human expert response**
+No — not necessarily, and in the described process the two are decoupled.
+The passenger's belongings go through the X-ray on the conveyor belt while the passenger separately goes through the millimeter wave scanner or metal detector. These are parallel streams, so a passenger can reach the post-X-ray belt to collect bags before, at roughly the same time as, or after finishing the body scan, depending on the relative service times of the two streams and any queueing at each.
+In practice the body scan (plus possible pat-down in Zone D) is often the longer or more variable step, so many passengers arrive at the belt and wait for their bags, but the reverse also occurs. The process does not enforce a fixed ordering between body-scan completion and belt arrival.
+## Exchange 2
+**Modeling Agent question**
+On a busy morning, which step causes most of the piling up?
+**Human expert response**
+On a busy morning, the bottleneck is almost always the **X-ray/bag-screening stream and the downstream Zone D secondary screening**, not the ID check or the body scanner itself.
+Reasons: the X-ray conveyor is a single shared resource per lane with a long, variable service time (bins, laptops, liquids, flagged items), and any bag flagged for additional search pulls a security officer off the line, creating a compounding slowdown. Body scanning is comparatively fast and parallelizable across lanes. ID check is quick and rarely the constraint.
+So the piling up concentrates at the **queue feeding the X-ray lanes (Zone B) and at the post-X-ray belt**, where passengers wait for their belongings — with secondary screening (Zone D) as the main source of variance. This is an empirical judgment based on typical checkpoint behavior, not a precise measured value.
+## Exchange 3
+**Modeling Agent question**
+Out of roughly 100 bags going through the X-ray, how many usually get flagged for a closer look?
+**Human expert response**
+Roughly 5–15 out of 100 bags, i.e. on the order of 10%, is the usual flag rate for X-ray secondary screening at a US checkpoint. This is an empirical judgment, not a precise measured value; the rate varies with the mix of passengers, the items carried, and how aggressively the operator is set to flag. Pre-Check bags tend to be flagged at a lower rate than regular-lane bags.
+## Exchange 4
+**Modeling Agent question**
+How many minutes does a closer manual inspection usually take?
+**Human expert response**
+Typically on the order of **1–3 minutes** for a routine manual bag inspection, with a central estimate around **2 minutes**. Simple re-scans or a quick swab are faster (under a minute); a full unpack-and-search, explosives-trace swab, or a pat-down can run **3–5 minutes or more**. The distribution is right-skewed, so a small fraction of inspections take much longer and drive most of the variance. This is an empirical judgment, not a precise measured value.
+## Exchange 5
+**Modeling Agent question**
+How many passengers, one after another, can one open lane screen per hour?
+**Human expert response**
+Roughly **100–200 passengers per hour per open lane**, with a central estimate around **150/hour** for a regular lane under normal conditions. This is an empirical judgment, not a precise measured value.
+The range reflects real-world variation: a well-staffed lane with few flagged bags and experienced passengers can approach 200/hour, while a lane slowed by heavy bin use, many laptops/liquids, frequent secondary screening, or Pre-Check-style mixed flow can drop toward 100/hour or below. Pre-Check lanes run higher (often 200–300/hour) because passengers divest less and are flagged less often.
+## Exchange 6
+**Modeling Agent question**
+How many passengers reach the checkpoint in a minute during a busy morning?
+**Human expert response**
+Roughly **10–30 passengers per minute** arriving at a single checkpoint during a busy morning peak, with a central estimate around **15–20/minute**. This is an empirical judgment, not a precise measured value.
+The range reflects real-world variation: a large hub checkpoint at peak can approach 30/minute, while a smaller or moderately busy checkpoint runs nearer 10/minute. Note this is the *arrival* rate; it should be compared against lane capacity (roughly 150/hour per lane, i.e. ~2.5/minute per lane) to see how many lanes must be open to keep the queue stable.
+## Exchange 7
+**Modeling Agent question**
+Of all passengers using a checkpoint on a typical day, what share is in Pre-Check?
+**Human expert response**
+Roughly **40–50%**, with a central estimate around **45%** — the problem statement itself cites about 45% enrollment in Pre-Check. This is an empirical judgment for a typical US checkpoint; the actual share varies by airport and time of day, and is often lower at smaller airports and higher at large hubs with many frequent/business travelers.
+## Exchange 8
+**Modeling Agent question**
+When the line grows long, do most travelers switch to an open lane?
+**Human expert response**
+No — most travelers do not switch lanes when the line grows long.
+In a standard checkpoint, passengers commit to a lane once they enter the Zone B queue feeding a specific screening line; the physical layout (railings, single-file queue, belongings already on the belt) makes switching impractical or impossible. Travelers generally stay in their chosen lane and wait.
+Switching mainly happens at the earlier stage — when a passenger is choosing which lane to join — and even then most people pick the nearest or shortest-looking queue and stay. The social norm against "cutting" (noted in the problem) further discourages mid-queue lane changes. So a long line mostly lengthens waiting rather than redistributing passengers across open lanes. This is an empirical judgment, not a measured value.
+## Exchange 9
+**Modeling Agent question**
+Do people tend to bring more bags and bins into the screening lane?
+**Human expert response**
+Yes — most passengers bring multiple items into the lane, not just one bag.
+Typical travelers arrive with a carry-on plus a personal item (purse, backpack, laptop bag), and each of those plus the divested items (shoes, belt, jacket, electronics, liquids, laptop) goes into its own bin. So a single passenger commonly occupies **2–4 bins** on the belt, and a family or a heavy traveler can occupy considerably more.
+This matters because bin count, not passenger count, is what loads the X-ray conveyor: more bins per passenger means longer belt occupancy and slower effective throughput per lane. Pre-Check passengers use fewer bins (no shoe/belt/jacket removal, laptop stays in bag), which is a large part of why their lanes run faster. This is an empirical judgment, not a measured value.
+## Exchange 10
+**Modeling Agent question**
+How long does checking one traveler's ID and boarding pass usually take?
+**Human expert response**
+Typically on the order of **10–20 seconds** per traveler for a routine ID and boarding-pass check, with a central estimate around **15 seconds**. This is an empirical judgment, not a precise measured value.
+The range reflects real-world variation: a quick glance-and-wave for a familiar or Pre-Check traveler can be under 10 seconds, while a slower check (document scrutiny, questions, a traveler fumbling for documents, or a flagged boarding pass) can run 30 seconds or more. It is one of the fastest steps in the checkpoint and rarely the bottleneck.
+</t>
+        </is>
+      </c>
+      <c r="L59" s="5" t="n">
+        <v>1734</v>
+      </c>
+      <c r="M59" s="6" t="n">
+        <v>16.09</v>
+      </c>
+      <c r="N59" s="4" t="n">
+        <v>0.7124999999999999</v>
+      </c>
+      <c r="O59" s="4" t="n">
+        <v>0.6697362038348276</v>
+      </c>
+      <c r="P59" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r2p2_20261003_160723</t>
+        </is>
+      </c>
+      <c r="Q59" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r2p2_20261003_160723/output/results/solution_report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Mechanism-Constraint-Parameter with Anti-Prescriptive Guard</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>interaction_workflow_c83b67c63c37</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>2024_C</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G60" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>What causes the biggest swings in control between players during a hard-fought tennis match?</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>Q1: What causes the biggest swings in control between players during a hard-fought tennis match?
+Q2: What stops a player's run of form in a tennis match, and around how long do such runs usually last?
+Q3: In tiebreaks on grass, about how often does the point's server win it, compared to normal games?
+Q4: What is the one physical limit that most often causes a player's game to collapse mid-match?
+Q5: What single on-court sign most reliably tells a coach that the flow is about to swing to the other player?
+Q6: What is the main limit on what a coach can change during a tennis match, while play is underway?
+Q7: How many points in a row does a player typically need to win to truly "take over" a tennis match's flow?
+Q8: What first-serve percentage is typical for a top player on grass, and how far does it drop when struggling?
+Q9: In a big-match flow swing, is it mostly physical fatigue or mostly mental/psychological, in your experience?
+Q10: After a player takes a big swing, how long does the new "hot hand" usually last before fading?</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>A1: The biggest swings in control in a hard-fought tennis match are driven mainly by **breaks of serve and the service game itself**, because the server wins roughly 60–80% of points (higher on fast surfaces, lower on clay). A single break — often decided by one or two points at 30–40 or deuce — flips game and set score and produces the largest measurable shift in who is favored.
+Secondary drivers, in rough order of impact:
+- **Clutch points** (break points, set points, tiebreaks): converting or squandering these changes both score and psychological edge disproportionately.
+- **Error/winner clusters**: a run of unforced errors or a burst of winners/aces over several points, not one point.
+- **Serving first vs. receiving pressure**: losing a set after being broken late, or a double fault at a critical moment.
+- **Physical/fatigue and time between points**: longer rallies and accumulated distance run erode the server's advantage in later sets.
+Note: whether these runs exceed what random point-by-point variation would produce is exactly the question the model must test — the above are the candidate mechanisms, not proof of momentum.
+A2: A run usually ends through one of these: the player's own **serve game ending** (a break, or simply rotating to receive), a **cluster of unforced errors or double faults**, a **successful opponent adjustment** (return position, target, tempo), or **physical/fatigue drift** in longer rallies and later sets. Clutch points — break points, deuce, tiebreaks — are where runs most often break, since the opponent raises risk there.
+On length: in point terms, runs of consecutive points by one player typically last only a handful of points — commonly **2–5**, occasionally reaching 6–8; runs beyond about 8–10 consecutive points are rare and usually coincide with a lopsided set or a serving mismatch. In game terms, a "run" is usually **one to two games**, rarely three or more. These are empirical judgments from match data, not fixed constants, and the key test is whether observed run lengths exceed what independent point outcomes would produce.
+A3: On grass, the tiebreak server wins roughly **65–75%** of tiebreak points — noticeably higher than the ~60–65% typical of normal grass service points, and higher than the ~62–68% average across surfaces.
+The reason is structural, not a different skill: in a tiebreak every point is a service point (no receiving games), and the server still holds the usual grass serve advantage, so the aggregate server win rate reflects pure serving strength rather than being diluted by return games. First-serve points in tiebreaks on grass commonly sit around 70–80%, second-serve points around 50–55%.
+These are empirical judgments from serve statistics, not fixed constants; the exact figure varies with the individual servers and how clutch the points are.
+A4: The single physical limit that most often causes a mid-match collapse is **aerobic/energy depletion — the depletion of glycogen and the onset of fatigue in long, physically demanding matches**, especially in later sets and after extended rallies.
+On grass this is somewhat muted (shorter points, faster holds), but in a hard-fought five-setter the decisive physical failure is typically **cumulative fatigue reducing first-step quickness and serve/return quality**, which shows up as a cluster of unforced errors, double faults, and lost break points. Heat and hydration accelerate it; it is an empirical judgment, not a fixed threshold.
+A5: The single most reliable on-court sign is a **drop in first-serve percentage and first-step quickness in the player who currently holds the flow** — visible as more second serves, shorter/defensive returns, and a cluster of unforced errors or double faults over a few points.
+Why this one: it is the earliest observable marker that the server's structural advantage (the main driver of control) is eroding, and it typically precedes the break rather than following it. Break points and deuce are where the swing is *confirmed*, but they are the symptom; the serve/quickness decline is the leading indicator.
+Caveat: it is a probabilistic sign, not deterministic — it raises the odds of a swing but does not guarantee one, and it is an empirical judgment from match observation, not a fixed threshold.
+A6: The main limit is **the rules and the clock**: a coach cannot stop play, call a timeout, or directly intervene during points or games. In-match coaching is confined to the short changeovers (about 90 seconds) and set breaks (about 120 seconds), plus brief player-initiated exchanges — and at Wimbledon 2023, off-court coaching was permitted only from the stands, not on court.
+So what a coach can change mid-match is limited to **verbal instruction and tactical adjustment** delivered in those windows: target selection, return position, serve patterns, tempo, and encouragement. Everything else — technique, fitness, stroke mechanics, equipment — is effectively fixed once the match starts. The practical constraint is therefore not the coach's knowledge but the **few, short, fixed communication windows** and the player's ability to absorb and execute changes under fatigue and pressure.
+A7: There is no fixed number, but empirically a player typically needs to win roughly **4–6 consecutive points** (or about **two consecutive games**, including a break) before the flow visibly shifts. Runs of 2–3 points are common noise; 4–6 points spanning a break or a hold-to-love is where control becomes apparent. Beyond ~8–10 consecutive points the shift is decisive, but such runs are rare and usually reflect a lopsided set or serving mismatch rather than a distinct "takeover." This is an empirical judgment, not a constant, and the real test is whether observed runs exceed what independent point outcomes would produce.
+A8: Typical first-serve percentage for a top player on grass is roughly **60–70%** for a match, with elite servers often in the **65–70%** range. On grass the serve is favored, so good servers tend to sit at the upper end.
+When struggling, first-serve percentage commonly drops to about **45–55%**, i.e. a fall of roughly **10–15 percentage points** from the player's norm. A drop into the low 40s or below is a clear sign of trouble — more second serves, more return pressure, and a higher break risk.
+These are empirical judgments from serve statistics, not fixed constants; the exact figures vary by player, opponent return quality, and match conditions.
+A9: Mostly **mental/psychological**, with physical fatigue as a secondary amplifier rather than the primary cause.
+In a big-match flow swing, the decisive factor is usually **psychological**: a lost clutch point (break point, set point, tiebreak), a double fault, or a squandered lead triggers a shift in confidence, risk tolerance, and decision-making — the player tightens, plays safer or over-hits, and the opponent gains belief. That psychological turn typically precedes the visible physical decline.
+Physical fatigue matters, but it usually **accelerates or exposes** an already-fragile mental state rather than initiating the swing. In a long five-setter, fatigue lowers first-serve percentage and first-step quickness, which then feeds the psychological spiral — but the swing itself is generally triggered by the mental event.
+Caveat: the two are entangled and hard to separate in observation; this is an empirical judgment, not a measured split.
+A10: Empirically, the new "hot hand" usually lasts only a short while — typically **one to two games, or roughly 4–8 points**, before it fades. The most common pattern is that the run carries through the remainder of the current game and the next one, then normalizes.
+Why it fades: the structural advantage rotates with the serve (the player must eventually receive), the opponent adjusts, and the psychological edge decays as the same clutch situations recur. Runs extending beyond about two games or ~8–10 points are uncommon and usually reflect a genuine serving or level mismatch rather than a transient hot hand.
+This is an empirical judgment from match observation, not a fixed constant; the real test is whether the post-swing run length exceeds what independent point outcomes would produce.</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Human Expert Dialogue
+## Exchange 1
+**Modeling Agent question**
+What causes the biggest swings in control between players during a hard-fought tennis match?
+**Human expert response**
+The biggest swings in control in a hard-fought tennis match are driven mainly by **breaks of serve and the service game itself**, because the server wins roughly 60–80% of points (higher on fast surfaces, lower on clay). A single break — often decided by one or two points at 30–40 or deuce — flips game and set score and produces the largest measurable shift in who is favored.
+Secondary drivers, in rough order of impact:
+- **Clutch points** (break points, set points, tiebreaks): converting or squandering these changes both score and psychological edge disproportionately.
+- **Error/winner clusters**: a run of unforced errors or a burst of winners/aces over several points, not one point.
+- **Serving first vs. receiving pressure**: losing a set after being broken late, or a double fault at a critical moment.
+- **Physical/fatigue and time between points**: longer rallies and accumulated distance run erode the server's advantage in later sets.
+Note: whether these runs exceed what random point-by-point variation would produce is exactly the question the model must test — the above are the candidate mechanisms, not proof of momentum.
+## Exchange 2
+**Modeling Agent question**
+What stops a player's run of form in a tennis match, and around how long do such runs usually last?
+**Human expert response**
+A run usually ends through one of these: the player's own **serve game ending** (a break, or simply rotating to receive), a **cluster of unforced errors or double faults**, a **successful opponent adjustment** (return position, target, tempo), or **physical/fatigue drift** in longer rallies and later sets. Clutch points — break points, deuce, tiebreaks — are where runs most often break, since the opponent raises risk there.
+On length: in point terms, runs of consecutive points by one player typically last only a handful of points — commonly **2–5**, occasionally reaching 6–8; runs beyond about 8–10 consecutive points are rare and usually coincide with a lopsided set or a serving mismatch. In game terms, a "run" is usually **one to two games**, rarely three or more. These are empirical judgments from match data, not fixed constants, and the key test is whether observed run lengths exceed what independent point outcomes would produce.
+## Exchange 3
+**Modeling Agent question**
+In tiebreaks on grass, about how often does the point's server win it, compared to normal games?
+**Human expert response**
+On grass, the tiebreak server wins roughly **65–75%** of tiebreak points — noticeably higher than the ~60–65% typical of normal grass service points, and higher than the ~62–68% average across surfaces.
+The reason is structural, not a different skill: in a tiebreak every point is a service point (no receiving games), and the server still holds the usual grass serve advantage, so the aggregate server win rate reflects pure serving strength rather than being diluted by return games. First-serve points in tiebreaks on grass commonly sit around 70–80%, second-serve points around 50–55%.
+These are empirical judgments from serve statistics, not fixed constants; the exact figure varies with the individual servers and how clutch the points are.
+## Exchange 4
+**Modeling Agent question**
+What is the one physical limit that most often causes a player's game to collapse mid-match?
+**Human expert response**
+The single physical limit that most often causes a mid-match collapse is **aerobic/energy depletion — the depletion of glycogen and the onset of fatigue in long, physically demanding matches**, especially in later sets and after extended rallies.
+On grass this is somewhat muted (shorter points, faster holds), but in a hard-fought five-setter the decisive physical failure is typically **cumulative fatigue reducing first-step quickness and serve/return quality**, which shows up as a cluster of unforced errors, double faults, and lost break points. Heat and hydration accelerate it; it is an empirical judgment, not a fixed threshold.
+## Exchange 5
+**Modeling Agent question**
+What single on-court sign most reliably tells a coach that the flow is about to swing to the other player?
+**Human expert response**
+The single most reliable on-court sign is a **drop in first-serve percentage and first-step quickness in the player who currently holds the flow** — visible as more second serves, shorter/defensive returns, and a cluster of unforced errors or double faults over a few points.
+Why this one: it is the earliest observable marker that the server's structural advantage (the main driver of control) is eroding, and it typically precedes the break rather than following it. Break points and deuce are where the swing is *confirmed*, but they are the symptom; the serve/quickness decline is the leading indicator.
+Caveat: it is a probabilistic sign, not deterministic — it raises the odds of a swing but does not guarantee one, and it is an empirical judgment from match observation, not a fixed threshold.
+## Exchange 6
+**Modeling Agent question**
+What is the main limit on what a coach can change during a tennis match, while play is underway?
+**Human expert response**
+The main limit is **the rules and the clock**: a coach cannot stop play, call a timeout, or directly intervene during points or games. In-match coaching is confined to the short changeovers (about 90 seconds) and set breaks (about 120 seconds), plus brief player-initiated exchanges — and at Wimbledon 2023, off-court coaching was permitted only from the stands, not on court.
+So what a coach can change mid-match is limited to **verbal instruction and tactical adjustment** delivered in those windows: target selection, return position, serve patterns, tempo, and encouragement. Everything else — technique, fitness, stroke mechanics, equipment — is effectively fixed once the match starts. The practical constraint is therefore not the coach's knowledge but the **few, short, fixed communication windows** and the player's ability to absorb and execute changes under fatigue and pressure.
+## Exchange 7
+**Modeling Agent question**
+How many points in a row does a player typically need to win to truly "take over" a tennis match's flow?
+**Human expert response**
+There is no fixed number, but empirically a player typically needs to win roughly **4–6 consecutive points** (or about **two consecutive games**, including a break) before the flow visibly shifts. Runs of 2–3 points are common noise; 4–6 points spanning a break or a hold-to-love is where control becomes apparent. Beyond ~8–10 consecutive points the shift is decisive, but such runs are rare and usually reflect a lopsided set or serving mismatch rather than a distinct "takeover." This is an empirical judgment, not a constant, and the real test is whether observed runs exceed what independent point outcomes would produce.
+## Exchange 8
+**Modeling Agent question**
+What first-serve percentage is typical for a top player on grass, and how far does it drop when struggling?
+**Human expert response**
+Typical first-serve percentage for a top player on grass is roughly **60–70%** for a match, with elite servers often in the **65–70%** range. On grass the serve is favored, so good servers tend to sit at the upper end.
+When struggling, first-serve percentage commonly drops to about **45–55%**, i.e. a fall of roughly **10–15 percentage points** from the player's norm. A drop into the low 40s or below is a clear sign of trouble — more second serves, more return pressure, and a higher break risk.
+These are empirical judgments from serve statistics, not fixed constants; the exact figures vary by player, opponent return quality, and match conditions.
+## Exchange 9
+**Modeling Agent question**
+In a big-match flow swing, is it mostly physical fatigue or mostly mental/psychological, in your experience?
+**Human expert response**
+Mostly **mental/psychological**, with physical fatigue as a secondary amplifier rather than the primary cause.
+In a big-match flow swing, the decisive factor is usually **psychological**: a lost clutch point (break point, set point, tiebreak), a double fault, or a squandered lead triggers a shift in confidence, risk tolerance, and decision-making — the player tightens, plays safer or over-hits, and the opponent gains belief. That psychological turn typically precedes the visible physical decline.
+Physical fatigue matters, but it usually **accelerates or exposes** an already-fragile mental state rather than initiating the swing. In a long five-setter, fatigue lowers first-serve percentage and first-step quickness, which then feeds the psychological spiral — but the swing itself is generally triggered by the mental event.
+Caveat: the two are entangled and hard to separate in observation; this is an empirical judgment, not a measured split.
+## Exchange 10
+**Modeling Agent question**
+After a player takes a big swing, how long does the new "hot hand" usually last before fading?
+**Human expert response**
+Empirically, the new "hot hand" usually lasts only a short while — typically **one to two games, or roughly 4–8 points**, before it fades. The most common pattern is that the run carries through the remainder of the current game and the next one, then normalizes.
+Why it fades: the structural advantage rotates with the serve (the player must eventually receive), the opponent adjusts, and the psychological edge decays as the same clutch situations recur. Runs extending beyond about two games or ~8–10 points are uncommon and usually reflect a genuine serving or level mismatch rather than a transient hot hand.
+This is an empirical judgment from match observation, not a fixed constant; the real test is whether the post-swing run length exceeds what independent point outcomes would produce.
+</t>
+        </is>
+      </c>
+      <c r="L60" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="M60" s="6" t="n">
+        <v>16.78</v>
+      </c>
+      <c r="N60" s="4" t="n">
+        <v>0.6291666666666668</v>
+      </c>
+      <c r="O60" s="4" t="n">
+        <v>0.6108203627035746</v>
+      </c>
+      <c r="P60" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r1p3_20261003_160723</t>
+        </is>
+      </c>
+      <c r="Q60" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r1p3_20261003_160723/output/results/solution_report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Mechanism-Constraint-Parameter with Anti-Prescriptive Guard</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>interaction_workflow_c83b67c63c37</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>2024_C</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F61" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G61" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>In Grand Slam tennis, when the flow of play swings from one player to the other mid-match, is the swing usually driven by the leading player's play changing, or by the other player's play changing?</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Q1: In Grand Slam tennis, when the flow of play swings from one player to the other mid-match, is the swing usually driven by the leading player's play changing, or by the other player's play changing?
+Q2: When a trailing player starts hitting better returns and winning more points, what is the main limit that stops them from turning that pressure into games?
+Q3: When a player serving under heavy break-point pressure gets pulled back, what is the main thing that breaks their serving first?
+Q4: A player who loses a long run of points usually bounces back how many points into the next rally?
+Q5: After a player breaks serve for the first time in a set, how often does the set follow that player?
+Q6: In a tense tennis game, are shifts in who is on top usually visible in the points right before they happen?
+Q7: During a five-set Grand Slam match, in which part of a set do players most often start to run out?
+Q8: In long matches, does a much younger player usually hold their level better, or does experience matter more in the late sets?
+Q9: On grass, does a strong first serve matter more or less for holding serve than on clay?
+Q10: Are patterns where one player takes over the match after a swing similar in table tennis as in tennis?</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>A1: Neither dominates: in Grand Slam tennis, mid-match swings are usually **mutual and asymmetric in cause** — the player who was behind typically raises level (or changes tactics) while the leader simultaneously drops level, and the two reinforce each other.
+Empirically, the more reliable driver is a **change by the player who is losing**: increased return aggression, higher first-serve percentage, fewer unforced errors, or a tactical adjustment (e.g., targeting a weaker wing, changing serve direction). The leader's apparent decline is often partly a *consequence* — facing better returns and more pressure, they take fewer risks, serve less freely, and their error rate rises.
+So the honest answer: the swing is usually initiated by the trailing player's play changing, with the leader's play changing in response. Pure one-sided explanations (only the leader "choking" or only the trailer "raising level") are the exception, not the rule. This is an empirical judgment, not a precise measured figure.
+A2: The main limit is **the serve-hold structure itself**: in men's Grand Slam tennis the server wins roughly 80% of service games, so a returning player who improves still has to convert a small number of break-point chances against a server who is, on average, favored in every point.
+Concretely, the trailing player's improved returning raises pressure but does not change the fact that:
+- they only get break chances on a minority of points, and those chances are often saved by a good first serve;
+- a single lost break point resets the game, and the opponent then serves out the next game comfortably;
+- the trailing player must also hold their own serve throughout, so any lapse on their own service game cancels the gain.
+So the pressure converts into games only if the improved returning is sustained across multiple return games and paired with holding serve — otherwise it produces points and deuce games, not breaks. This is an empirical regularity, not a precise figure.
+A3: The main thing that breaks a server's first serve under break-point pressure is **loss of rhythm and margin on the first delivery itself** — the server starts steering the ball rather than swinging freely, so first-serve percentage drops and second serves become the norm.
+Concretely, the pressure causes the server to:
+- aim closer to lines or hit a safer, slower first serve, both of which reduce the percentage in;
+- rush the motion (tighter arm, earlier contact), producing more faults;
+- then face the returner from a second serve, where the returner is far more aggressive.
+So the first serve breaks first because it is the shot most sensitive to tension and the one the server consciously tries to control. Once the first serve is gone, the whole game structure collapses toward the returner. This is an empirical regularity, not a precise figure.
+A4: There is no fixed number — a bounce-back is not reliably tied to a specific point count. Empirically, the recovery is usually **immediate or near-immediate**: the player who just lost a long run most often wins the very next point or within the next one to two points, because the run-ending point itself is typically where the opponent's level regresses (a missed first serve, an error) rather than a deliberate reset by the trailing player.
+But this is a weak tendency, not a rule. Long runs frequently end on a *server's* point (a good first serve or an ace), which is not a genuine "bounce back" by the player who was losing the run. So the honest answer: expect the run to break within roughly the next 1–3 points, but do not treat any specific point index as a reliable indicator. This is an empirical judgment, not a measured figure.
+A5: Not reliably — breaking first in a set is a modest advantage, not a decisive one.
+Empirically, the player who breaks first in a set goes on to win that set somewhat more often than not, but the edge is small — roughly in the 55–65% range in men's Grand Slam play, and it varies with the quality gap between the players. The reason it is not higher: the opponent immediately gets a chance to break back, and a single break is often neutralized before the set ends.
+So the honest answer: usually the set follows the first breaker, but only slightly more often than a coin flip, and the effect is much weaker than the "first break decides the set" intuition suggests. This is an empirical judgment, not a precise measured figure.
+A6: No — usually not in a reliable, visible way.
+Empirically, the points immediately before a shift look much like ordinary points: the player about to lose the edge often still wins a point or two, and the player about to take over often still makes errors. The shift is typically only identifiable *after* it has occurred, once a run of points or a break has already happened.
+What is sometimes visible just before a swing is not the outcome of points but a *change in process*: first-serve percentage dipping, more second serves faced, longer rallies, more unforced errors, or a player suddenly going for more on returns. These are weak, noisy precursors — they raise the probability of a swing slightly but do not announce it.
+So the honest answer: shifts are mostly not visible in the points right before they happen; at best, subtle changes in serve/error patterns give a faint early signal. This is an empirical judgment, not a measured figure.
+A7: Late in the set — specifically **after the 4th–5th game and especially from around 4–4 onward**, and most acutely in the **closing games of the set** (games 8–12, including tiebreaks).
+The pattern: players are freshest at the start of a set, and the physical and mental cost accumulates across the set. The heaviest fatigue shows in:
+- long deuce games and long rallies late in the set;
+- the game immediately after a long game (the "letdown" game);
+- tiebreaks, where concentration and leg drive are most taxed.
+Across a five-set match, this compounds — the deepest fatigue appears in the **4th and 5th sets**, and within those sets the late-set games are where running out is most visible. Note this is an empirical judgment about a general tendency, not a measured figure; individual fitness, match duration, and rally length shift it considerably.
+A8: In long matches, **youth usually holds physical level better, but experience matters more in the decisive late-set moments** — and the two act on different things.
+- **Physical level (running, rally tolerance, serve speed late):** the younger player generally holds up better, especially in the 4th and 5th sets and in long deuce games. This is the clearest youth advantage.
+- **Point-level and game-level execution under pressure (break points, tiebreaks, serving out sets):** experience usually matters more. Older players more often manage tension, choose better patterns, and avoid the error clusters that youth produces when fatigued.
+So the honest answer: youth tends to win the *physical* late-match battle, experience tends to win the *decision and pressure* battle. Which dominates depends on the gap in age and the gap in big-match experience — a large age gap with similar experience favors youth; similar age with a large experience gap favors the veteran. This is an empirical judgment, not a measured figure.
+A9: More — a strong first serve matters **more** for holding serve on grass than on clay.
+On grass the ball skids and stays low, the bounce is faster and less predictable, and the returner has less time to react. That makes a good first serve disproportionately valuable: free points and weak returns are easier to come by, so servers who land a high percentage of first serves hold at a higher rate than on any other surface. Grass also rewards the serve-and-first-ball pattern, so the serve's value extends into the point it sets up.
+On clay the ball sits up and the surface is slower, giving the returner time to play the ball back and neutralizing raw serve speed; rallies lengthen and holds are harder, so the serve alone decides less.
+So: on grass the first serve is the single most important hold-preserving shot; on clay it is still important but far less decisive. This is an empirical regularity, not a precise figure.
+A10: Broadly yes, but with important differences in magnitude and mechanism.
+Similar: table tennis shows the same qualitative phenomena — runs of points, momentum-like swings, server advantage (though smaller than tennis), and the trailing player often initiating a swing by raising aggression or changing serve/receive tactics. Long runs and "taking over" a match after a swing are common and recognizable.
+Different: the serve-hold structure that dominates tennis does not exist in table tennis. Serves alternate every two points and the server's edge is modest, so a swing converts into games/sets far more easily — there is no "hold" barrier limiting the trailing player. Points are also much shorter and faster, so swings happen quicker and runs are shorter in point count but more frequent. Fatigue and five-set endurance dynamics have no real analogue.
+So the *pattern* (a swing, then one player taking over) transfers; the *rate and ease* of conversion do not. This is an empirical judgment, not a measured figure.</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Human Expert Dialogue
+## Exchange 1
+**Modeling Agent question**
+In Grand Slam tennis, when the flow of play swings from one player to the other mid-match, is the swing usually driven by the leading player's play changing, or by the other player's play changing?
+**Human expert response**
+Neither dominates: in Grand Slam tennis, mid-match swings are usually **mutual and asymmetric in cause** — the player who was behind typically raises level (or changes tactics) while the leader simultaneously drops level, and the two reinforce each other.
+Empirically, the more reliable driver is a **change by the player who is losing**: increased return aggression, higher first-serve percentage, fewer unforced errors, or a tactical adjustment (e.g., targeting a weaker wing, changing serve direction). The leader's apparent decline is often partly a *consequence* — facing better returns and more pressure, they take fewer risks, serve less freely, and their error rate rises.
+So the honest answer: the swing is usually initiated by the trailing player's play changing, with the leader's play changing in response. Pure one-sided explanations (only the leader "choking" or only the trailer "raising level") are the exception, not the rule. This is an empirical judgment, not a precise measured figure.
+## Exchange 2
+**Modeling Agent question**
+When a trailing player starts hitting better returns and winning more points, what is the main limit that stops them from turning that pressure into games?
+**Human expert response**
+The main limit is **the serve-hold structure itself**: in men's Grand Slam tennis the server wins roughly 80% of service games, so a returning player who improves still has to convert a small number of break-point chances against a server who is, on average, favored in every point.
+Concretely, the trailing player's improved returning raises pressure but does not change the fact that:
+- they only get break chances on a minority of points, and those chances are often saved by a good first serve;
+- a single lost break point resets the game, and the opponent then serves out the next game comfortably;
+- the trailing player must also hold their own serve throughout, so any lapse on their own service game cancels the gain.
+So the pressure converts into games only if the improved returning is sustained across multiple return games and paired with holding serve — otherwise it produces points and deuce games, not breaks. This is an empirical regularity, not a precise figure.
+## Exchange 3
+**Modeling Agent question**
+When a player serving under heavy break-point pressure gets pulled back, what is the main thing that breaks their serving first?
+**Human expert response**
+The main thing that breaks a server's first serve under break-point pressure is **loss of rhythm and margin on the first delivery itself** — the server starts steering the ball rather than swinging freely, so first-serve percentage drops and second serves become the norm.
+Concretely, the pressure causes the server to:
+- aim closer to lines or hit a safer, slower first serve, both of which reduce the percentage in;
+- rush the motion (tighter arm, earlier contact), producing more faults;
+- then face the returner from a second serve, where the returner is far more aggressive.
+So the first serve breaks first because it is the shot most sensitive to tension and the one the server consciously tries to control. Once the first serve is gone, the whole game structure collapses toward the returner. This is an empirical regularity, not a precise figure.
+## Exchange 4
+**Modeling Agent question**
+A player who loses a long run of points usually bounces back how many points into the next rally?
+**Human expert response**
+There is no fixed number — a bounce-back is not reliably tied to a specific point count. Empirically, the recovery is usually **immediate or near-immediate**: the player who just lost a long run most often wins the very next point or within the next one to two points, because the run-ending point itself is typically where the opponent's level regresses (a missed first serve, an error) rather than a deliberate reset by the trailing player.
+But this is a weak tendency, not a rule. Long runs frequently end on a *server's* point (a good first serve or an ace), which is not a genuine "bounce back" by the player who was losing the run. So the honest answer: expect the run to break within roughly the next 1–3 points, but do not treat any specific point index as a reliable indicator. This is an empirical judgment, not a measured figure.
+## Exchange 5
+**Modeling Agent question**
+After a player breaks serve for the first time in a set, how often does the set follow that player?
+**Human expert response**
+Not reliably — breaking first in a set is a modest advantage, not a decisive one.
+Empirically, the player who breaks first in a set goes on to win that set somewhat more often than not, but the edge is small — roughly in the 55–65% range in men's Grand Slam play, and it varies with the quality gap between the players. The reason it is not higher: the opponent immediately gets a chance to break back, and a single break is often neutralized before the set ends.
+So the honest answer: usually the set follows the first breaker, but only slightly more often than a coin flip, and the effect is much weaker than the "first break decides the set" intuition suggests. This is an empirical judgment, not a precise measured figure.
+## Exchange 6
+**Modeling Agent question**
+In a tense tennis game, are shifts in who is on top usually visible in the points right before they happen?
+**Human expert response**
+No — usually not in a reliable, visible way.
+Empirically, the points immediately before a shift look much like ordinary points: the player about to lose the edge often still wins a point or two, and the player about to take over often still makes errors. The shift is typically only identifiable *after* it has occurred, once a run of points or a break has already happened.
+What is sometimes visible just before a swing is not the outcome of points but a *change in process*: first-serve percentage dipping, more second serves faced, longer rallies, more unforced errors, or a player suddenly going for more on returns. These are weak, noisy precursors — they raise the probability of a swing slightly but do not announce it.
+So the honest answer: shifts are mostly not visible in the points right before they happen; at best, subtle changes in serve/error patterns give a faint early signal. This is an empirical judgment, not a measured figure.
+## Exchange 7
+**Modeling Agent question**
+During a five-set Grand Slam match, in which part of a set do players most often start to run out?
+**Human expert response**
+Late in the set — specifically **after the 4th–5th game and especially from around 4–4 onward**, and most acutely in the **closing games of the set** (games 8–12, including tiebreaks).
+The pattern: players are freshest at the start of a set, and the physical and mental cost accumulates across the set. The heaviest fatigue shows in:
+- long deuce games and long rallies late in the set;
+- the game immediately after a long game (the "letdown" game);
+- tiebreaks, where concentration and leg drive are most taxed.
+Across a five-set match, this compounds — the deepest fatigue appears in the **4th and 5th sets**, and within those sets the late-set games are where running out is most visible. Note this is an empirical judgment about a general tendency, not a measured figure; individual fitness, match duration, and rally length shift it considerably.
+## Exchange 8
+**Modeling Agent question**
+In long matches, does a much younger player usually hold their level better, or does experience matter more in the late sets?
+**Human expert response**
+In long matches, **youth usually holds physical level better, but experience matters more in the decisive late-set moments** — and the two act on different things.
+- **Physical level (running, rally tolerance, serve speed late):** the younger player generally holds up better, especially in the 4th and 5th sets and in long deuce games. This is the clearest youth advantage.
+- **Point-level and game-level execution under pressure (break points, tiebreaks, serving out sets):** experience usually matters more. Older players more often manage tension, choose better patterns, and avoid the error clusters that youth produces when fatigued.
+So the honest answer: youth tends to win the *physical* late-match battle, experience tends to win the *decision and pressure* battle. Which dominates depends on the gap in age and the gap in big-match experience — a large age gap with similar experience favors youth; similar age with a large experience gap favors the veteran. This is an empirical judgment, not a measured figure.
+## Exchange 9
+**Modeling Agent question**
+On grass, does a strong first serve matter more or less for holding serve than on clay?
+**Human expert response**
+More — a strong first serve matters **more** for holding serve on grass than on clay.
+On grass the ball skids and stays low, the bounce is faster and less predictable, and the returner has less time to react. That makes a good first serve disproportionately valuable: free points and weak returns are easier to come by, so servers who land a high percentage of first serves hold at a higher rate than on any other surface. Grass also rewards the serve-and-first-ball pattern, so the serve's value extends into the point it sets up.
+On clay the ball sits up and the surface is slower, giving the returner time to play the ball back and neutralizing raw serve speed; rallies lengthen and holds are harder, so the serve alone decides less.
+So: on grass the first serve is the single most important hold-preserving shot; on clay it is still important but far less decisive. This is an empirical regularity, not a precise figure.
+## Exchange 10
+**Modeling Agent question**
+Are patterns where one player takes over the match after a swing similar in table tennis as in tennis?
+**Human expert response**
+Broadly yes, but with important differences in magnitude and mechanism.
+Similar: table tennis shows the same qualitative phenomena — runs of points, momentum-like swings, server advantage (though smaller than tennis), and the trailing player often initiating a swing by raising aggression or changing serve/receive tactics. Long runs and "taking over" a match after a swing are common and recognizable.
+Different: the serve-hold structure that dominates tennis does not exist in table tennis. Serves alternate every two points and the server's edge is modest, so a swing converts into games/sets far more easily — there is no "hold" barrier limiting the trailing player. Points are also much shorter and faster, so swings happen quicker and runs are shorter in point count but more frequent. Fatigue and five-set endurance dynamics have no real analogue.
+So the *pattern* (a swing, then one player taking over) transfers; the *rate and ease* of conversion do not. This is an empirical judgment, not a measured figure.
+</t>
+        </is>
+      </c>
+      <c r="L61" s="5" t="n">
+        <v>2619</v>
+      </c>
+      <c r="M61" s="6" t="n">
+        <v>18.06</v>
+      </c>
+      <c r="N61" s="4" t="n">
+        <v>0.6791666666666667</v>
+      </c>
+      <c r="O61" s="4" t="n">
+        <v>0.6108203627035746</v>
+      </c>
+      <c r="P61" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r2p3_20261003_160723</t>
+        </is>
+      </c>
+      <c r="Q61" s="3" t="inlineStr">
+        <is>
+          <t>/public1/home/stu52275901007/workspace/ghj_workspace/ModelingAgent/openclaw_experiments/evolve_exp/claude_fp8_scratch_ten_5r/cpe_evaluations/round_10/train_candidate/runs/round_10/r2p3_20261003_160723/output/results/solution_report.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q55"/>
+  <autoFilter ref="A1:Q61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12662,7 +13872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13169,8 +14379,51 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Mechanism-Constraint-Parameter with Anti-Prescriptive Guard</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 15:22:04</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 16:41:25</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>79.34729396666667</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>43.78315168333334</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>1.474348333333333</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>34.03104775</v>
+      </c>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>run.json开始时间 + 工件mtime结束时间</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K11"/>
+  <autoFilter ref="A1:K12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>